<commit_message>
Updated all files with quarterly prices
</commit_message>
<xml_diff>
--- a/MU.xlsx
+++ b/MU.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MyStockData/Finance-StockLists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EDF1D7A-0AB3-9D4F-9B5C-E47F5A81603E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B012DCA-618F-7848-B37D-0ED948A5F98F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" activeTab="2" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -15155,11 +15155,11 @@
     <v>Powered by Refinitiv</v>
     <v>1255</v>
     <v>103.38</v>
-    <v>2.1964000000000001</v>
-    <v>-4.25</v>
-    <v>-4.9810000000000002E-3</v>
-    <v>-4.95</v>
-    <v>-5.8309999999999994E-3</v>
+    <v>2.2547000000000001</v>
+    <v>-51.63</v>
+    <v>-5.9028999999999998E-2</v>
+    <v>-6.53</v>
+    <v>-7.9340000000000001E-3</v>
     <v>USD</v>
     <v>Micron Technology, Inc. provides memory and storage solutions. The Company delivers a portfolio of high-performance dynamic random-access memory (DRAM), NAND, and NOR memory and storage products through its Micron and Crucial brands. The Company's products enable advancing in artificial intelligence (AI) and compute-intensive applications. Its segments include Cloud Memory Business Unit (CMBU), Core Data Center Business Unit (CDBU), Mobile and Client Business Unit (MCBU) and Automotive and Embedded Business Unit (AEBU). CMBU is focused on memory solutions for large hyperscale cloud customers, and high bandwidth memory (HBM) for all data center customers. CDBU is focused on memory solutions for mid-tier cloud, enterprise, and OEM data center customers and storage solutions for all data center customers. MCBU is focused on memory and storage solutions for mobile and client segments. AEBU is focused on memory and storage solutions for the automotive, industrial, and consumer segments.</v>
     <v>53000</v>
@@ -15167,25 +15167,25 @@
     <v>XNAS</v>
     <v>XNAS</v>
     <v>8000 S Federal Way, Po Box 6, BOISE, ID, 83716-9632 US</v>
-    <v>903.96</v>
+    <v>930.88</v>
     <v>Semiconductors &amp; Semiconductor Equipment</v>
     <v>Stock</v>
-    <v>46220.99999732578</v>
+    <v>46234.909704015627</v>
     <v>0</v>
-    <v>804</v>
-    <v>958798187350</v>
+    <v>818</v>
+    <v>929524320790</v>
     <v>MICRON TECHNOLOGY, INC.</v>
     <v>MICRON TECHNOLOGY, INC.</v>
-    <v>822.52499999999998</v>
-    <v>19.3154</v>
-    <v>853.2</v>
-    <v>848.95</v>
-    <v>844</v>
+    <v>919.65</v>
+    <v>18.632300000000001</v>
+    <v>874.66</v>
+    <v>823.03</v>
+    <v>816.5</v>
     <v>1129393000</v>
     <v>MU</v>
     <v>MICRON TECHNOLOGY, INC. (XNAS:MU)</v>
-    <v>63346278</v>
-    <v>51936325</v>
+    <v>54184317</v>
+    <v>50529428</v>
     <v>1984</v>
   </rv>
   <rv s="2">
@@ -15207,19 +15207,19 @@
     <v>268435456</v>
     <v>1</v>
     <v>Powered by Refinitiv</v>
-    <v>46.87</v>
+    <v>47.14</v>
     <v>39.47</v>
-    <v>-0.28000000000000003</v>
-    <v>-6.1279999999999998E-3</v>
+    <v>0.41</v>
+    <v>8.8710000000000004E-3</v>
     <v>US</v>
-    <v>45.5</v>
+    <v>46.86</v>
     <v>Index</v>
     <v>3</v>
-    <v>45.11</v>
+    <v>46.51</v>
     <v>10 Y TSY YLD NDX</v>
-    <v>45.21</v>
-    <v>45.69</v>
-    <v>45.41</v>
+    <v>46.69</v>
+    <v>46.22</v>
+    <v>46.63</v>
     <v>TNX</v>
     <v>10 Y TSY YLD NDX</v>
   </rv>
@@ -15441,9 +15441,9 @@
       <v>at close</v>
       <v>from previous close</v>
       <v>from previous close</v>
-      <v>Source: Nasdaq</v>
+      <v>Source: Nasdaq Last Sale</v>
       <v>GMT</v>
-      <v>Delayed 15 minutes</v>
+      <v>Real-Time Nasdaq Last Sale</v>
       <v>from close</v>
       <v>from close</v>
     </spb>
@@ -16040,7 +16040,7 @@
       </c>
       <c r="F3" s="191">
         <f ca="1">Statement!AC153</f>
-        <v>972896.70000000007</v>
+        <v>943192.38</v>
       </c>
       <c r="H3" s="189" t="str">
         <f>'AVG target price'!B5</f>
@@ -16048,7 +16048,7 @@
       </c>
       <c r="I3" s="215">
         <f ca="1">'AVG target price'!C5</f>
-        <v>556.76821664507384</v>
+        <v>541.23797874688739</v>
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.2">
@@ -16064,7 +16064,7 @@
       </c>
       <c r="F4" s="192">
         <f ca="1">Statement!AC154</f>
-        <v>948490.70000000007</v>
+        <v>918786.38</v>
       </c>
       <c r="H4" s="189" t="str">
         <f>'AVG target price'!B6</f>
@@ -16072,7 +16072,7 @@
       </c>
       <c r="I4" s="215">
         <f ca="1">'AVG target price'!C6</f>
-        <v>539.08850228373342</v>
+        <v>530.53040027865063</v>
       </c>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.2">
@@ -16081,7 +16081,7 @@
       </c>
       <c r="C5" s="212" cm="1">
         <f t="array" aca="1" ref="C5" ca="1">_FV(C3,"Price",TRUE)</f>
-        <v>848.95</v>
+        <v>823.03</v>
       </c>
       <c r="E5" s="189" t="s">
         <v>248</v>
@@ -16096,7 +16096,7 @@
       </c>
       <c r="I5" s="215">
         <f ca="1">'AVG target price'!C7</f>
-        <v>175.74882789862582</v>
+        <v>172.82666091307053</v>
       </c>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.2">
@@ -16105,14 +16105,14 @@
       </c>
       <c r="C6" s="212" cm="1">
         <f t="array" aca="1" ref="C6" ca="1">_FV(C3,"Price (Extended hours)",TRUE)</f>
-        <v>844</v>
+        <v>816.5</v>
       </c>
       <c r="E6" s="189" t="s">
         <v>242</v>
       </c>
       <c r="F6" s="194">
         <f ca="1">Statement!AC150</f>
-        <v>19.220058863482002</v>
+        <v>18.633235227529998</v>
       </c>
       <c r="H6" s="189" t="str">
         <f>'AVG target price'!B8</f>
@@ -16120,7 +16120,7 @@
       </c>
       <c r="I6" s="215">
         <f ca="1">'AVG target price'!C8</f>
-        <v>815.34470379949528</v>
+        <v>802.24085036536019</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -16129,14 +16129,14 @@
       </c>
       <c r="C7" s="6" cm="1">
         <f t="array" aca="1" ref="C7" ca="1">_FV(C3,"Change")</f>
-        <v>-4.25</v>
+        <v>-51.63</v>
       </c>
       <c r="E7" s="190" t="s">
         <v>201</v>
       </c>
       <c r="F7" s="195">
         <f ca="1">Statement!AC151</f>
-        <v>10.711323858475309</v>
+        <v>10.384287502492413</v>
       </c>
       <c r="H7" s="188" t="str">
         <f>'AVG target price'!B9</f>
@@ -16144,7 +16144,7 @@
       </c>
       <c r="I7" s="216">
         <f ca="1">'AVG target price'!C9</f>
-        <v>521.73756265673217</v>
+        <v>511.70897257599222</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
@@ -16153,14 +16153,14 @@
       </c>
       <c r="C8" s="6" cm="1">
         <f t="array" aca="1" ref="C8" ca="1">_FV(C3,"Change (extended hours)",TRUE)</f>
-        <v>-4.95</v>
+        <v>-6.53</v>
       </c>
       <c r="E8" s="189" t="s">
         <v>270</v>
       </c>
       <c r="F8" s="196">
         <f ca="1">Statement!AC161</f>
-        <v>2.5663567365373938E-2</v>
+        <v>2.6471799952412677E-2</v>
       </c>
       <c r="H8" s="188" t="str">
         <f>'AVG target price'!B11</f>
@@ -16168,7 +16168,7 @@
       </c>
       <c r="I8" s="217">
         <f ca="1">'AVG target price'!C11</f>
-        <v>-0.38543193043555907</v>
+        <v>-0.37826206508147669</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -16177,14 +16177,14 @@
       </c>
       <c r="C9" s="73" cm="1">
         <f t="array" aca="1" ref="C9" ca="1">_FV(C3,"Change (%)",TRUE)</f>
-        <v>-4.9810000000000002E-3</v>
+        <v>-5.9028999999999998E-2</v>
       </c>
       <c r="E9" s="189" t="s">
         <v>293</v>
       </c>
       <c r="F9" s="196">
         <f ca="1">Statement!AC162</f>
-        <v>5.2028976971553093E-2</v>
+        <v>5.3667545532969638E-2</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
@@ -16193,21 +16193,21 @@
       </c>
       <c r="C10" s="73" cm="1">
         <f t="array" aca="1" ref="C10" ca="1">_FV(C3,"Change % (extended hours)",TRUE)</f>
-        <v>-5.8309999999999994E-3</v>
+        <v>-7.9340000000000001E-3</v>
       </c>
       <c r="E10" s="189" t="s">
         <v>298</v>
       </c>
       <c r="F10" s="196">
         <f ca="1">Statement!AC164</f>
-        <v>1.1532570724106679E-3</v>
+        <v>1.1895770404760904E-3</v>
       </c>
       <c r="H10" s="188" t="s">
         <v>376</v>
       </c>
       <c r="I10" s="216">
         <f ca="1">DDM!C26</f>
-        <v>4.2276451228905545</v>
+        <v>4.0900488180775083</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
@@ -16223,7 +16223,7 @@
       </c>
       <c r="F11" s="197">
         <f ca="1">Statement!AC163</f>
-        <v>6.2430060663172158E-4</v>
+        <v>6.4396194549408892E-4</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
@@ -16248,7 +16248,7 @@
       </c>
       <c r="C13" s="213" cm="1">
         <f t="array" aca="1" ref="C13" ca="1">_FV(C3,"Beta")</f>
-        <v>2.1964000000000001</v>
+        <v>2.2547000000000001</v>
       </c>
       <c r="E13" s="189" t="s">
         <v>104</v>
@@ -16264,7 +16264,7 @@
       </c>
       <c r="C14" s="214" cm="1">
         <f t="array" aca="1" ref="C14" ca="1">_FV(C3,"Volume average",TRUE)</f>
-        <v>51936325</v>
+        <v>50529428</v>
       </c>
       <c r="E14" s="190" t="s">
         <v>105</v>
@@ -16280,7 +16280,7 @@
       </c>
       <c r="F15" s="196">
         <f ca="1">Statement!AC176</f>
-        <v>2.5085910970815296E-2</v>
+        <v>2.5875951203083298E-2</v>
       </c>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.2">
@@ -16390,7 +16390,7 @@
       </c>
       <c r="F26" s="223" cm="1">
         <f t="array" aca="1" ref="F26" ca="1">_FV(E26,"Price")</f>
-        <v>45.41</v>
+        <v>46.63</v>
       </c>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.2">
@@ -16405,7 +16405,7 @@
       </c>
       <c r="F27" s="224">
         <f ca="1">F26/1000</f>
-        <v>4.5409999999999999E-2</v>
+        <v>4.6630000000000005E-2</v>
       </c>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
@@ -22594,7 +22594,7 @@
       </c>
       <c r="C6" s="137">
         <f ca="1">Overview!C5</f>
-        <v>848.95</v>
+        <v>823.03</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22603,7 +22603,7 @@
       </c>
       <c r="C7" s="138">
         <f ca="1">C5*C6</f>
-        <v>972896.70000000007</v>
+        <v>943192.38</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22621,7 +22621,7 @@
       </c>
       <c r="C9" s="139">
         <f ca="1">Overview!F27</f>
-        <v>4.5409999999999999E-2</v>
+        <v>4.6630000000000005E-2</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22630,7 +22630,7 @@
       </c>
       <c r="C10" s="137">
         <f ca="1">Overview!C13</f>
-        <v>2.1964000000000001</v>
+        <v>2.2547000000000001</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22673,7 +22673,7 @@
       </c>
       <c r="C16" s="46">
         <f ca="1">C8/(C8+C7)</f>
-        <v>5.847016820749491E-3</v>
+        <v>6.0300487805865057E-3</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22682,7 +22682,7 @@
       </c>
       <c r="C17" s="46">
         <f ca="1">C7/(C8+C7)</f>
-        <v>0.99415298317925049</v>
+        <v>0.99396995121941345</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22700,7 +22700,7 @@
       </c>
       <c r="C19" s="46">
         <f ca="1">C9+C10*C11</f>
-        <v>0.14424799999999999</v>
+        <v>0.14809149999999999</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22709,7 +22709,7 @@
       </c>
       <c r="C20" s="46">
         <f ca="1">(C17*C19)+(C16*C18)</f>
-        <v>0.1436401558253485</v>
+        <v>0.14744145169637959</v>
       </c>
     </row>
   </sheetData>
@@ -22960,7 +22960,7 @@
       </c>
       <c r="L8" s="130">
         <f ca="1">L7*(1+C14)/(C15-C14)</f>
-        <v>674669.97257515765</v>
+        <v>656010.24401870964</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -23014,23 +23014,23 @@
       <c r="G10" s="142"/>
       <c r="H10" s="130">
         <f ca="1">H7/(1+$C$15)^H9</f>
-        <v>37926.629988255299</v>
+        <v>37800.984935286942</v>
       </c>
       <c r="I10" s="130">
         <f t="shared" ref="I10:L10" ca="1" si="0">I7/(1+$C$15)^I9</f>
-        <v>54044.725991947998</v>
+        <v>53687.235510816361</v>
       </c>
       <c r="J10" s="130">
         <f t="shared" ca="1" si="0"/>
-        <v>67631.200846602602</v>
+        <v>66961.270042211356</v>
       </c>
       <c r="K10" s="130">
         <f t="shared" ca="1" si="0"/>
-        <v>63555.565265369965</v>
+        <v>62717.542152575195</v>
       </c>
       <c r="L10" s="130">
         <f t="shared" ca="1" si="0"/>
-        <v>45631.001527711087</v>
+        <v>44880.150725935142</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -23049,7 +23049,7 @@
       <c r="K11" s="141"/>
       <c r="L11" s="130">
         <f ca="1">L8/(1+C15)^L9</f>
-        <v>344861.2526553676</v>
+        <v>329805.54027710791</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.2">
@@ -23072,7 +23072,7 @@
       </c>
       <c r="C15" s="139">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>0.1436401558253485</v>
+        <v>0.14744145169637959</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
@@ -23087,7 +23087,7 @@
       </c>
       <c r="C19" s="64">
         <f ca="1">SUM(H10:L10)</f>
-        <v>268789.12361988699</v>
+        <v>266047.18336682499</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.2">
@@ -23096,7 +23096,7 @@
       </c>
       <c r="C20" s="64">
         <f ca="1">L11</f>
-        <v>344861.2526553676</v>
+        <v>329805.54027710791</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
@@ -23105,7 +23105,7 @@
       </c>
       <c r="C21" s="94">
         <f ca="1">C19+C20</f>
-        <v>613650.37627525465</v>
+        <v>595852.72364393296</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
@@ -23132,7 +23132,7 @@
       </c>
       <c r="C24" s="94">
         <f ca="1">C21+C22-C23</f>
-        <v>638056.37627525465</v>
+        <v>620258.72364393296</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.2">
@@ -23150,7 +23150,7 @@
       </c>
       <c r="C26" s="146">
         <f ca="1">C24/C25</f>
-        <v>556.76821664507384</v>
+        <v>541.23797874688739</v>
       </c>
     </row>
   </sheetData>
@@ -24159,7 +24159,7 @@
       </c>
       <c r="C39" s="139">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>0.1436401558253485</v>
+        <v>0.14744145169637959</v>
       </c>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.2">
@@ -24185,7 +24185,7 @@
       </c>
       <c r="C42" s="24">
         <f ca="1">C41/(1+C39)^5-G30+G31</f>
-        <v>593389.42361715843</v>
+        <v>583581.83871933364</v>
       </c>
     </row>
     <row r="43" spans="2:14" x14ac:dyDescent="0.2">
@@ -24212,7 +24212,7 @@
       </c>
       <c r="C45" s="24">
         <f ca="1">C42+C43-C44</f>
-        <v>617795.42361715843</v>
+        <v>607987.83871933364</v>
       </c>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.2">
@@ -24230,7 +24230,7 @@
       </c>
       <c r="C47" s="146">
         <f ca="1">C45/C46</f>
-        <v>539.08850228373342</v>
+        <v>530.53040027865063</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.2">
@@ -24254,7 +24254,7 @@
       </c>
       <c r="C51" s="139">
         <f ca="1">IF(Overview!C29&gt;0,Overview!C29,WACC!C19)</f>
-        <v>0.14424799999999999</v>
+        <v>0.14809149999999999</v>
       </c>
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.2">
@@ -24289,7 +24289,7 @@
       </c>
       <c r="C55" s="146">
         <f ca="1">C54/(1+C51)^5</f>
-        <v>175.74882789862582</v>
+        <v>172.82666091307053</v>
       </c>
     </row>
     <row r="57" spans="2:3" x14ac:dyDescent="0.2">
@@ -24313,7 +24313,7 @@
       </c>
       <c r="C59" s="139">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>0.1436401558253485</v>
+        <v>0.14744145169637959</v>
       </c>
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.2">
@@ -24339,7 +24339,7 @@
       </c>
       <c r="C62" s="24">
         <f ca="1">C61/(1+C59)^5-G30+G31</f>
-        <v>909979.03055422159</v>
+        <v>894962.01451870275</v>
       </c>
     </row>
     <row r="63" spans="2:3" x14ac:dyDescent="0.2">
@@ -24366,7 +24366,7 @@
       </c>
       <c r="C65" s="24">
         <f ca="1">C62+C63-C64</f>
-        <v>934385.03055422159</v>
+        <v>919368.01451870275</v>
       </c>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.2">
@@ -24384,7 +24384,7 @@
       </c>
       <c r="C67" s="146">
         <f ca="1">C65/C66</f>
-        <v>815.34470379949528</v>
+        <v>802.24085036536019</v>
       </c>
     </row>
   </sheetData>
@@ -24448,7 +24448,7 @@
       </c>
       <c r="C5" s="137">
         <f ca="1">DCF!C26</f>
-        <v>556.76821664507384</v>
+        <v>541.23797874688739</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -24457,7 +24457,7 @@
       </c>
       <c r="C6" s="137">
         <f ca="1">Multiples!C47</f>
-        <v>539.08850228373342</v>
+        <v>530.53040027865063</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -24466,7 +24466,7 @@
       </c>
       <c r="C7" s="137">
         <f ca="1">Multiples!C55</f>
-        <v>175.74882789862582</v>
+        <v>172.82666091307053</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -24475,7 +24475,7 @@
       </c>
       <c r="C8" s="137">
         <f ca="1">Multiples!C67</f>
-        <v>815.34470379949528</v>
+        <v>802.24085036536019</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -24484,7 +24484,7 @@
       </c>
       <c r="C9" s="146">
         <f ca="1">AVERAGE(C5:C8)</f>
-        <v>521.73756265673217</v>
+        <v>511.70897257599222</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -24493,7 +24493,7 @@
       </c>
       <c r="C10" s="137">
         <f ca="1">Overview!C5</f>
-        <v>848.95</v>
+        <v>823.03</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -24502,7 +24502,7 @@
       </c>
       <c r="C11" s="158">
         <f ca="1">(C9-C10)/C10</f>
-        <v>-0.38543193043555907</v>
+        <v>-0.37826206508147669</v>
       </c>
     </row>
   </sheetData>
@@ -24972,7 +24972,7 @@
       </c>
       <c r="C24" s="139">
         <f ca="1">IF(Overview!C29&gt;0,Overview!C29,WACC!C19)</f>
-        <v>0.14424799999999999</v>
+        <v>0.14809149999999999</v>
       </c>
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.2">
@@ -24989,7 +24989,7 @@
       </c>
       <c r="C26" s="146">
         <f ca="1">C23/(C24-C25)</f>
-        <v>4.2276451228905545</v>
+        <v>4.0900488180775083</v>
       </c>
     </row>
   </sheetData>
@@ -25226,7 +25226,7 @@
       <c r="K8" s="141"/>
       <c r="L8" s="130">
         <f ca="1">L7*(1+C20)/(C21-C20)</f>
-        <v>1458553.1018510824</v>
+        <v>1418213.0747681747</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -25280,23 +25280,23 @@
       <c r="G10" s="142"/>
       <c r="H10" s="130">
         <f ca="1">H7/(1+$C$21)^H9</f>
-        <v>6136.2990890618439</v>
+        <v>6115.9704802633933</v>
       </c>
       <c r="I10" s="130">
         <f t="shared" ref="I10:L10" ca="1" si="1">I7/(1+$C$21)^I9</f>
-        <v>12287.190898618286</v>
+        <v>12205.914627798489</v>
       </c>
       <c r="J10" s="130">
         <f t="shared" ca="1" si="1"/>
-        <v>24603.60194114496</v>
+        <v>24359.887344434803</v>
       </c>
       <c r="K10" s="130">
         <f t="shared" ca="1" si="1"/>
-        <v>49265.713658472036</v>
+        <v>48616.111903822479</v>
       </c>
       <c r="L10" s="130">
         <f t="shared" ca="1" si="1"/>
-        <v>98648.586011289095</v>
+        <v>97025.339371487469</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -25315,7 +25315,7 @@
       <c r="K11" s="141"/>
       <c r="L11" s="130">
         <f ca="1">L8/(1+C21)^L9</f>
-        <v>745547.40868166124</v>
+        <v>712998.81917489739</v>
       </c>
     </row>
     <row r="13" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
@@ -25331,7 +25331,7 @@
       </c>
       <c r="C15" s="160">
         <f ca="1">Overview!C5</f>
-        <v>848.95</v>
+        <v>823.03</v>
       </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.2">
@@ -25340,7 +25340,7 @@
       </c>
       <c r="C16" s="160">
         <f ca="1">C36</f>
-        <v>851.10256889304469</v>
+        <v>819.95397954181055</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -25379,7 +25379,7 @@
       </c>
       <c r="C21" s="226">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>0.1436401558253485</v>
+        <v>0.14744145169637959</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.2">
@@ -25397,7 +25397,7 @@
       </c>
       <c r="C23" s="165">
         <f ca="1">C15*C22</f>
-        <v>958464.55</v>
+        <v>929200.87</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.2">
@@ -25424,7 +25424,7 @@
       </c>
       <c r="C26" s="166">
         <f ca="1">C23+C25-C24</f>
-        <v>934058.55</v>
+        <v>904794.87</v>
       </c>
     </row>
     <row r="27" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
@@ -25440,7 +25440,7 @@
       </c>
       <c r="C29" s="165">
         <f ca="1">SUM(H10:L10)</f>
-        <v>190941.39159858623</v>
+        <v>188323.22372780665</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
@@ -25449,7 +25449,7 @@
       </c>
       <c r="C30" s="165">
         <f ca="1">L11</f>
-        <v>745547.40868166124</v>
+        <v>712998.81917489739</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
@@ -25458,7 +25458,7 @@
       </c>
       <c r="C31" s="168">
         <f ca="1">C29+C30</f>
-        <v>936488.80028024747</v>
+        <v>901322.0429027041</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
@@ -25485,7 +25485,7 @@
       </c>
       <c r="C34" s="168">
         <f ca="1">C31+C32-C33</f>
-        <v>960894.80028024747</v>
+        <v>925728.0429027041</v>
       </c>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.2">
@@ -25503,7 +25503,7 @@
       </c>
       <c r="C36" s="171">
         <f ca="1">C34/C35</f>
-        <v>851.10256889304469</v>
+        <v>819.95397954181055</v>
       </c>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.2">
@@ -32541,17 +32541,33 @@
       <c r="Q116" s="63">
         <v>122</v>
       </c>
-      <c r="T116" s="68"/>
-      <c r="U116" s="68"/>
-      <c r="V116" s="68"/>
-      <c r="W116" s="68"/>
-      <c r="X116" s="68"/>
-      <c r="Y116" s="68"/>
-      <c r="Z116" s="68"/>
-      <c r="AA116" s="68"/>
+      <c r="T116" s="63">
+        <v>95.57</v>
+      </c>
+      <c r="U116" s="63">
+        <v>97.7</v>
+      </c>
+      <c r="V116" s="63">
+        <v>91.82</v>
+      </c>
+      <c r="W116" s="63">
+        <v>96.55</v>
+      </c>
+      <c r="X116" s="63">
+        <v>122</v>
+      </c>
+      <c r="Y116" s="63">
+        <v>230.26</v>
+      </c>
+      <c r="Z116" s="63">
+        <v>415.56</v>
+      </c>
+      <c r="AA116" s="63">
+        <v>923.52</v>
+      </c>
       <c r="AC116" s="63">
         <f ca="1">Overview!C5</f>
-        <v>848.95</v>
+        <v>823.03</v>
       </c>
     </row>
     <row r="117" spans="1:31" x14ac:dyDescent="0.2">
@@ -32588,17 +32604,41 @@
         <f>Q116/Q85</f>
         <v>122</v>
       </c>
-      <c r="T117" s="68"/>
-      <c r="U117" s="68"/>
-      <c r="V117" s="68"/>
-      <c r="W117" s="68"/>
-      <c r="X117" s="68"/>
-      <c r="Y117" s="68"/>
-      <c r="Z117" s="68"/>
-      <c r="AA117" s="68"/>
+      <c r="T117" s="65">
+        <f t="shared" ref="T117:AA117" si="74">T116/T85</f>
+        <v>95.57</v>
+      </c>
+      <c r="U117" s="65">
+        <f t="shared" si="74"/>
+        <v>97.7</v>
+      </c>
+      <c r="V117" s="65">
+        <f t="shared" si="74"/>
+        <v>91.82</v>
+      </c>
+      <c r="W117" s="65">
+        <f t="shared" si="74"/>
+        <v>96.55</v>
+      </c>
+      <c r="X117" s="65">
+        <f t="shared" si="74"/>
+        <v>122</v>
+      </c>
+      <c r="Y117" s="65">
+        <f t="shared" si="74"/>
+        <v>230.26</v>
+      </c>
+      <c r="Z117" s="65">
+        <f t="shared" si="74"/>
+        <v>415.56</v>
+      </c>
+      <c r="AA117" s="65">
+        <f t="shared" si="74"/>
+        <v>923.52</v>
+      </c>
       <c r="AC117" s="65">
         <f ca="1">AC116/AC85</f>
-        <v>848.95</v>
+        <v>823.03</v>
       </c>
     </row>
     <row r="119" spans="1:31" x14ac:dyDescent="0.2">
@@ -32712,19 +32752,19 @@
         <v>102</v>
       </c>
       <c r="M123" s="76">
-        <f t="shared" ref="M123:P123" si="74">M121*M122</f>
+        <f t="shared" ref="M123:P123" si="75">M121*M122</f>
         <v>9.9593875851756192E-2</v>
       </c>
       <c r="N123" s="76">
-        <f t="shared" si="74"/>
+        <f t="shared" si="75"/>
         <v>0.1310592459605027</v>
       </c>
       <c r="O123" s="76">
-        <f t="shared" si="74"/>
+        <f t="shared" si="75"/>
         <v>-9.0780340523547179E-2</v>
       </c>
       <c r="P123" s="76">
-        <f t="shared" si="74"/>
+        <f t="shared" si="75"/>
         <v>1.1207790711075256E-2</v>
       </c>
       <c r="Q123" s="76">
@@ -32786,19 +32826,19 @@
         <v>104</v>
       </c>
       <c r="M125" s="76">
-        <f t="shared" ref="M125:P125" si="75">M123*M124</f>
+        <f t="shared" ref="M125:P125" si="76">M123*M124</f>
         <v>0.13340768898094826</v>
       </c>
       <c r="N125" s="76">
-        <f t="shared" si="75"/>
+        <f t="shared" si="76"/>
         <v>0.17406375859097922</v>
       </c>
       <c r="O125" s="76">
-        <f t="shared" si="75"/>
+        <f t="shared" si="76"/>
         <v>-0.13220761559383501</v>
       </c>
       <c r="P125" s="76">
-        <f t="shared" si="75"/>
+        <f t="shared" si="76"/>
         <v>1.7238705102922601E-2</v>
       </c>
       <c r="Q125" s="76">
@@ -32960,35 +33000,35 @@
       <c r="P131" s="49"/>
       <c r="Q131" s="49"/>
       <c r="T131" s="25">
-        <f t="shared" ref="T131:AA131" si="76">U5</f>
+        <f t="shared" ref="T131:AA131" si="77">U5</f>
         <v>8709</v>
       </c>
       <c r="U131" s="25">
-        <f t="shared" si="76"/>
+        <f t="shared" si="77"/>
         <v>8053</v>
       </c>
       <c r="V131" s="25">
-        <f t="shared" si="76"/>
+        <f t="shared" si="77"/>
         <v>9301</v>
       </c>
       <c r="W131" s="25">
-        <f t="shared" si="76"/>
+        <f t="shared" si="77"/>
         <v>11315</v>
       </c>
       <c r="X131" s="25">
-        <f t="shared" si="76"/>
+        <f t="shared" si="77"/>
         <v>13643</v>
       </c>
       <c r="Y131" s="25">
-        <f t="shared" si="76"/>
+        <f t="shared" si="77"/>
         <v>23860</v>
       </c>
       <c r="Z131" s="25">
-        <f t="shared" si="76"/>
+        <f t="shared" si="77"/>
         <v>41456</v>
       </c>
       <c r="AA131" s="25">
-        <f t="shared" si="76"/>
+        <f t="shared" si="77"/>
         <v>0</v>
       </c>
       <c r="AC131" s="49"/>
@@ -33013,31 +33053,31 @@
       <c r="P132" s="49"/>
       <c r="Q132" s="49"/>
       <c r="T132" s="229" t="str">
-        <f t="shared" ref="T132:Z132" si="77">IF(T131&gt;T130, "BEAT", IF(T131&lt;T129, "MISSED", "MET"))</f>
+        <f t="shared" ref="T132:Z132" si="78">IF(T131&gt;T130, "BEAT", IF(T131&lt;T129, "MISSED", "MET"))</f>
         <v>MET</v>
       </c>
       <c r="U132" s="229" t="str">
-        <f t="shared" si="77"/>
+        <f t="shared" si="78"/>
         <v>MET</v>
       </c>
       <c r="V132" s="229" t="str">
-        <f t="shared" si="77"/>
+        <f t="shared" si="78"/>
         <v>BEAT</v>
       </c>
       <c r="W132" s="229" t="str">
-        <f t="shared" si="77"/>
+        <f t="shared" si="78"/>
         <v>BEAT</v>
       </c>
       <c r="X132" s="229" t="str">
-        <f t="shared" si="77"/>
+        <f t="shared" si="78"/>
         <v>BEAT</v>
       </c>
       <c r="Y132" s="229" t="str">
-        <f t="shared" si="77"/>
+        <f t="shared" si="78"/>
         <v>BEAT</v>
       </c>
       <c r="Z132" s="229" t="str">
-        <f t="shared" si="77"/>
+        <f t="shared" si="78"/>
         <v>BEAT</v>
       </c>
       <c r="AA132" s="229" t="str">
@@ -33164,27 +33204,27 @@
         <v>1.41</v>
       </c>
       <c r="V135" s="65">
-        <f t="shared" ref="V135:AA135" si="78">W26</f>
+        <f t="shared" ref="V135:AA135" si="79">W26</f>
         <v>1.68</v>
       </c>
       <c r="W135" s="65">
-        <f t="shared" si="78"/>
+        <f t="shared" si="79"/>
         <v>2.83</v>
       </c>
       <c r="X135" s="65">
-        <f t="shared" si="78"/>
+        <f t="shared" si="79"/>
         <v>4.5999999999999996</v>
       </c>
       <c r="Y135" s="65">
-        <f t="shared" si="78"/>
+        <f t="shared" si="79"/>
         <v>12.07</v>
       </c>
       <c r="Z135" s="65">
-        <f t="shared" si="78"/>
+        <f t="shared" si="79"/>
         <v>24.67</v>
       </c>
       <c r="AA135" s="65">
-        <f t="shared" si="78"/>
+        <f t="shared" si="79"/>
         <v>0</v>
       </c>
       <c r="AC135" s="49"/>
@@ -33209,31 +33249,31 @@
       <c r="P136" s="49"/>
       <c r="Q136" s="49"/>
       <c r="T136" s="229" t="str">
-        <f t="shared" ref="T136:Z136" si="79">IF(T135&gt;T134, "BEAT", IF(T135&lt;T133, "MISSED", "MET"))</f>
+        <f t="shared" ref="T136:Z136" si="80">IF(T135&gt;T134, "BEAT", IF(T135&lt;T133, "MISSED", "MET"))</f>
         <v>MET</v>
       </c>
       <c r="U136" s="229" t="str">
-        <f t="shared" si="79"/>
+        <f t="shared" si="80"/>
         <v>MET</v>
       </c>
       <c r="V136" s="229" t="str">
-        <f t="shared" si="79"/>
+        <f t="shared" si="80"/>
         <v>BEAT</v>
       </c>
       <c r="W136" s="229" t="str">
-        <f t="shared" si="79"/>
+        <f t="shared" si="80"/>
         <v>BEAT</v>
       </c>
       <c r="X136" s="229" t="str">
-        <f t="shared" si="79"/>
+        <f t="shared" si="80"/>
         <v>BEAT</v>
       </c>
       <c r="Y136" s="229" t="str">
-        <f t="shared" si="79"/>
+        <f t="shared" si="80"/>
         <v>BEAT</v>
       </c>
       <c r="Z136" s="229" t="str">
-        <f t="shared" si="79"/>
+        <f t="shared" si="80"/>
         <v>BEAT</v>
       </c>
       <c r="AA136" s="229" t="str">
@@ -33326,55 +33366,55 @@
         <v>139</v>
       </c>
       <c r="M141" s="122">
-        <f t="shared" ref="M141:Q142" si="80">M30/M5*365</f>
+        <f t="shared" ref="M141:Q142" si="81">M30/M5*365</f>
         <v>69.969861035914093</v>
       </c>
       <c r="N141" s="122">
-        <f t="shared" si="80"/>
+        <f t="shared" si="81"/>
         <v>60.876845048442682</v>
       </c>
       <c r="O141" s="122">
-        <f t="shared" si="80"/>
+        <f t="shared" si="81"/>
         <v>57.380630630630634</v>
       </c>
       <c r="P141" s="122">
-        <f t="shared" si="80"/>
+        <f t="shared" si="81"/>
         <v>96.152084743737802</v>
       </c>
       <c r="Q141" s="122">
-        <f t="shared" si="80"/>
+        <f t="shared" si="81"/>
         <v>90.473674353898005</v>
       </c>
       <c r="T141" s="122">
-        <f t="shared" ref="T141:AA141" si="81">T30/T5*90</f>
+        <f t="shared" ref="T141:AA141" si="82">T30/T5*90</f>
         <v>76.819354838709671</v>
       </c>
       <c r="U141" s="122">
-        <f t="shared" si="81"/>
+        <f t="shared" si="82"/>
         <v>76.710299689975884</v>
       </c>
       <c r="V141" s="122">
-        <f t="shared" si="81"/>
+        <f t="shared" si="82"/>
         <v>72.688439091021976</v>
       </c>
       <c r="W141" s="122">
-        <f t="shared" si="81"/>
+        <f t="shared" si="82"/>
         <v>71.953553381356841</v>
       </c>
       <c r="X141" s="122">
-        <f t="shared" si="81"/>
+        <f t="shared" si="82"/>
         <v>73.694211224038895</v>
       </c>
       <c r="Y141" s="122">
-        <f t="shared" si="81"/>
+        <f t="shared" si="82"/>
         <v>67.181704903613578</v>
       </c>
       <c r="Z141" s="122">
-        <f t="shared" si="81"/>
+        <f t="shared" si="82"/>
         <v>65.30846605196983</v>
       </c>
       <c r="AA141" s="122">
-        <f t="shared" si="81"/>
+        <f t="shared" si="82"/>
         <v>67.354544577383251</v>
       </c>
       <c r="AC141" s="122">
@@ -33387,55 +33427,55 @@
         <v>140</v>
       </c>
       <c r="M142" s="122">
-        <f t="shared" si="80"/>
+        <f t="shared" si="81"/>
         <v>94.766520078694597</v>
       </c>
       <c r="N142" s="122">
-        <f t="shared" si="80"/>
+        <f t="shared" si="81"/>
         <v>144.24644128113877</v>
       </c>
       <c r="O142" s="122">
-        <f t="shared" si="80"/>
+        <f t="shared" si="81"/>
         <v>180.5411063930172</v>
       </c>
       <c r="P142" s="122">
-        <f t="shared" si="80"/>
+        <f t="shared" si="81"/>
         <v>166.13883475228226</v>
       </c>
       <c r="Q142" s="122">
-        <f t="shared" si="80"/>
+        <f t="shared" si="81"/>
         <v>135.5065540990891</v>
       </c>
       <c r="T142" s="122">
-        <f t="shared" ref="T142:AA142" si="82">T31/T6*365</f>
+        <f t="shared" ref="T142:AA142" si="83">T31/T6*365</f>
         <v>646.19489327747863</v>
       </c>
       <c r="U142" s="122">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>592.67394142883791</v>
       </c>
       <c r="V142" s="122">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>645.88506876227905</v>
       </c>
       <c r="W142" s="122">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>549.86276540652511</v>
       </c>
       <c r="X142" s="122">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>487.07474844274077</v>
       </c>
       <c r="Y142" s="122">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>499.38719359679845</v>
       </c>
       <c r="Z142" s="122">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>494.25962325962325</v>
       </c>
       <c r="AA142" s="122">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>488.58671874999999</v>
       </c>
       <c r="AC142" s="122">
@@ -33468,35 +33508,35 @@
         <v>156.4934459009109</v>
       </c>
       <c r="T143" s="122">
-        <f t="shared" ref="T143:AA143" si="83">T38/T6*90</f>
+        <f t="shared" ref="T143:AA143" si="84">T38/T6*90</f>
         <v>131.04129263913825</v>
       </c>
       <c r="U143" s="122">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>119.63066592053723</v>
       </c>
       <c r="V143" s="122">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>109.20235756385068</v>
       </c>
       <c r="W143" s="122">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>136.11082340756084</v>
       </c>
       <c r="X143" s="122">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>138.70148538572113</v>
       </c>
       <c r="Y143" s="122">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>146.60830415207604</v>
       </c>
       <c r="Z143" s="122">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>162.11793611793613</v>
       </c>
       <c r="AA143" s="122">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>218.26406250000002</v>
       </c>
       <c r="AC143" s="122">
@@ -33513,55 +33553,55 @@
         <v>52.271099318520285</v>
       </c>
       <c r="N144" s="122">
-        <f t="shared" ref="N144:Q144" si="84">N141+N142-N143</f>
+        <f t="shared" ref="N144:Q144" si="85">N141+N142-N143</f>
         <v>73.281649318905295</v>
       </c>
       <c r="O144" s="122">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>152.72062827158368</v>
       </c>
       <c r="P144" s="122">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>125.65459782200224</v>
       </c>
       <c r="Q144" s="122">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>69.486782552076193</v>
       </c>
       <c r="T144" s="122">
-        <f t="shared" ref="T144" si="85">T141+T142-T143</f>
+        <f t="shared" ref="T144" si="86">T141+T142-T143</f>
         <v>591.97295547705016</v>
       </c>
       <c r="U144" s="122">
-        <f t="shared" ref="U144" si="86">U141+U142-U143</f>
+        <f t="shared" ref="U144" si="87">U141+U142-U143</f>
         <v>549.75357519827651</v>
       </c>
       <c r="V144" s="122">
-        <f t="shared" ref="V144" si="87">V141+V142-V143</f>
+        <f t="shared" ref="V144" si="88">V141+V142-V143</f>
         <v>609.37115028945038</v>
       </c>
       <c r="W144" s="122">
-        <f t="shared" ref="W144" si="88">W141+W142-W143</f>
+        <f t="shared" ref="W144" si="89">W141+W142-W143</f>
         <v>485.70549538032117</v>
       </c>
       <c r="X144" s="122">
-        <f t="shared" ref="X144" si="89">X141+X142-X143</f>
+        <f t="shared" ref="X144" si="90">X141+X142-X143</f>
         <v>422.06747428105854</v>
       </c>
       <c r="Y144" s="122">
-        <f t="shared" ref="Y144" si="90">Y141+Y142-Y143</f>
+        <f t="shared" ref="Y144" si="91">Y141+Y142-Y143</f>
         <v>419.96059434833603</v>
       </c>
       <c r="Z144" s="122">
-        <f t="shared" ref="Z144:AA144" si="91">Z141+Z142-Z143</f>
+        <f t="shared" ref="Z144:AA144" si="92">Z141+Z142-Z143</f>
         <v>397.450153193657</v>
       </c>
       <c r="AA144" s="122">
-        <f t="shared" si="91"/>
+        <f t="shared" si="92"/>
         <v>337.67720082738322</v>
       </c>
       <c r="AC144" s="122">
-        <f t="shared" ref="AC144" si="92">AC141+AC142-AC143</f>
+        <f t="shared" ref="AC144" si="93">AC141+AC142-AC143</f>
         <v>22.941609834516981</v>
       </c>
     </row>
@@ -33590,35 +33630,35 @@
         <v>0.26912212683467185</v>
       </c>
       <c r="T145" s="122">
-        <f t="shared" ref="T145:AA145" si="93">T108/T49</f>
+        <f t="shared" ref="T145:AA145" si="94">T108/T49</f>
         <v>0.29684695663734462</v>
       </c>
       <c r="U145" s="122">
-        <f t="shared" si="93"/>
+        <f t="shared" si="94"/>
         <v>0.29457016475415093</v>
       </c>
       <c r="V145" s="122">
-        <f t="shared" si="93"/>
+        <f t="shared" si="94"/>
         <v>0.29516994633273702</v>
       </c>
       <c r="W145" s="122">
-        <f t="shared" si="93"/>
+        <f t="shared" si="94"/>
         <v>0.30623866950421691</v>
       </c>
       <c r="X145" s="122">
-        <f t="shared" si="93"/>
+        <f t="shared" si="94"/>
         <v>0.26912212683467185</v>
       </c>
       <c r="Y145" s="122">
-        <f t="shared" si="93"/>
+        <f t="shared" si="94"/>
         <v>0.19991157364894738</v>
       </c>
       <c r="Z145" s="122">
-        <f t="shared" si="93"/>
+        <f t="shared" si="94"/>
         <v>0.13996880994769456</v>
       </c>
       <c r="AA145" s="122">
-        <f t="shared" si="93"/>
+        <f t="shared" si="94"/>
         <v>5.6808704975973949E-2</v>
       </c>
       <c r="AC145" s="122">
@@ -33651,35 +33691,35 @@
         <v>4.8758423336102648E-2</v>
       </c>
       <c r="T146" s="183">
-        <f t="shared" ref="T146:AA146" si="94">(T108-T107)/T49</f>
+        <f t="shared" ref="T146:AA146" si="95">(T108-T107)/T49</f>
         <v>9.4059515632270496E-2</v>
       </c>
       <c r="U146" s="183">
-        <f t="shared" si="94"/>
+        <f t="shared" si="95"/>
         <v>0.10772058037908414</v>
       </c>
       <c r="V146" s="183">
-        <f t="shared" si="94"/>
+        <f t="shared" si="95"/>
         <v>9.7978738716509362E-2</v>
       </c>
       <c r="W146" s="183">
-        <f t="shared" si="94"/>
+        <f t="shared" si="95"/>
         <v>6.5578939071490497E-2</v>
       </c>
       <c r="X146" s="183">
-        <f t="shared" si="94"/>
+        <f t="shared" si="95"/>
         <v>4.8758423336102648E-2</v>
       </c>
       <c r="Y146" s="183">
-        <f t="shared" si="94"/>
+        <f t="shared" si="95"/>
         <v>-4.4043124851205658E-3</v>
       </c>
       <c r="Z146" s="183">
-        <f t="shared" si="94"/>
+        <f t="shared" si="95"/>
         <v>-8.9498889026897968E-2</v>
       </c>
       <c r="AA146" s="183">
-        <f t="shared" si="94"/>
+        <f t="shared" si="95"/>
         <v>-0.24230570668361065</v>
       </c>
       <c r="AC146" s="183">
@@ -33712,35 +33752,35 @@
         <v>1.8509690937663699</v>
       </c>
       <c r="T147" s="122">
-        <f t="shared" ref="T147:AA147" si="95">(T107+T30)/T40</f>
+        <f t="shared" ref="T147:AA147" si="96">(T107+T30)/T40</f>
         <v>1.704909169550173</v>
       </c>
       <c r="U147" s="122">
-        <f t="shared" si="95"/>
+        <f t="shared" si="96"/>
         <v>1.7933444259567388</v>
       </c>
       <c r="V147" s="122">
-        <f t="shared" si="95"/>
+        <f t="shared" si="96"/>
         <v>2.0431636409800684</v>
       </c>
       <c r="W147" s="122">
-        <f t="shared" si="95"/>
+        <f t="shared" si="96"/>
         <v>1.9387271830291071</v>
       </c>
       <c r="X147" s="122">
-        <f t="shared" si="95"/>
+        <f t="shared" si="96"/>
         <v>1.8509690937663699</v>
       </c>
       <c r="Y147" s="122">
-        <f t="shared" si="95"/>
+        <f t="shared" si="96"/>
         <v>1.8407131011608624</v>
       </c>
       <c r="Z147" s="122">
-        <f t="shared" si="95"/>
+        <f t="shared" si="96"/>
         <v>2.3741606043648571</v>
       </c>
       <c r="AA147" s="122">
-        <f t="shared" si="95"/>
+        <f t="shared" si="96"/>
         <v>3.1379823481116587</v>
       </c>
       <c r="AC147" s="122">
@@ -33773,35 +33813,35 @@
         <v>2.5179849834119086</v>
       </c>
       <c r="T148" s="122">
-        <f t="shared" ref="T148:AA148" si="96">T32/T40</f>
+        <f t="shared" ref="T148:AA148" si="97">T32/T40</f>
         <v>2.6353806228373702</v>
       </c>
       <c r="U148" s="122">
-        <f t="shared" si="96"/>
+        <f t="shared" si="97"/>
         <v>2.7169162506932891</v>
       </c>
       <c r="V148" s="122">
-        <f t="shared" si="96"/>
+        <f t="shared" si="97"/>
         <v>3.1343150945791547</v>
       </c>
       <c r="W148" s="122">
-        <f t="shared" si="96"/>
+        <f t="shared" si="97"/>
         <v>2.7547113961519485</v>
       </c>
       <c r="X148" s="122">
-        <f t="shared" si="96"/>
+        <f t="shared" si="97"/>
         <v>2.5179849834119086</v>
       </c>
       <c r="Y148" s="122">
-        <f t="shared" si="96"/>
+        <f t="shared" si="97"/>
         <v>2.4597844112769485</v>
       </c>
       <c r="Z148" s="122">
-        <f t="shared" si="96"/>
+        <f t="shared" si="97"/>
         <v>2.8968242865137102</v>
       </c>
       <c r="AA148" s="122">
-        <f t="shared" si="96"/>
+        <f t="shared" si="97"/>
         <v>3.4245176518883413</v>
       </c>
       <c r="AC148" s="122">
@@ -33834,35 +33874,35 @@
         <v>N/A</v>
       </c>
       <c r="T149" s="185">
-        <f t="shared" ref="T149:AA149" si="97">IF(T13&gt;=0,"N/A",IF(T12&lt;=0,"N/A",T12/-T13))</f>
+        <f t="shared" ref="T149:AA149" si="98">IF(T13&gt;=0,"N/A",IF(T12&lt;=0,"N/A",T12/-T13))</f>
         <v>304.39999999999998</v>
       </c>
       <c r="U149" s="185">
-        <f t="shared" si="97"/>
+        <f t="shared" si="98"/>
         <v>197.63636363636363</v>
       </c>
       <c r="V149" s="185">
-        <f t="shared" si="97"/>
+        <f t="shared" si="98"/>
         <v>443.25</v>
       </c>
       <c r="W149" s="185" t="str">
-        <f t="shared" si="97"/>
+        <f t="shared" si="98"/>
         <v>N/A</v>
       </c>
       <c r="X149" s="185" t="str">
-        <f t="shared" si="97"/>
+        <f t="shared" si="98"/>
         <v>N/A</v>
       </c>
       <c r="Y149" s="185" t="str">
-        <f t="shared" si="97"/>
+        <f t="shared" si="98"/>
         <v>N/A</v>
       </c>
       <c r="Z149" s="185" t="str">
-        <f t="shared" si="97"/>
+        <f t="shared" si="98"/>
         <v>N/A</v>
       </c>
       <c r="AA149" s="185" t="str">
-        <f t="shared" si="97"/>
+        <f t="shared" si="98"/>
         <v>N/A</v>
       </c>
       <c r="AC149" s="185" t="str">
@@ -33904,7 +33944,7 @@
       <c r="AA150" s="49"/>
       <c r="AC150" s="72">
         <f ca="1">AC117/Statement!AC26</f>
-        <v>19.220058863482002</v>
+        <v>18.633235227529998</v>
       </c>
     </row>
     <row r="151" spans="2:29" x14ac:dyDescent="0.2">
@@ -33941,7 +33981,7 @@
       <c r="AA151" s="49"/>
       <c r="AC151" s="72">
         <f ca="1">AC117/(Statement!AC5/Statement!AC22)</f>
-        <v>10.711323858475309</v>
+        <v>10.384287502492413</v>
       </c>
     </row>
     <row r="152" spans="2:29" x14ac:dyDescent="0.2">
@@ -33968,17 +34008,41 @@
         <f>Q117/(Statement!Q49/Statement!Q75)</f>
         <v>2.5271669897535309</v>
       </c>
-      <c r="T152" s="49"/>
-      <c r="U152" s="49"/>
-      <c r="V152" s="49"/>
-      <c r="W152" s="49"/>
-      <c r="X152" s="49"/>
-      <c r="Y152" s="49"/>
-      <c r="Z152" s="49"/>
-      <c r="AA152" s="49"/>
+      <c r="T152" s="72">
+        <f>T117/(Statement!T49/Statement!T75)</f>
+        <v>2.3484330061376881</v>
+      </c>
+      <c r="U152" s="72">
+        <f>U117/(Statement!U49/Statement!U75)</f>
+        <v>2.3257431031903755</v>
+      </c>
+      <c r="V152" s="72">
+        <f>V117/(Statement!V49/Statement!V75)</f>
+        <v>2.1108045977011494</v>
+      </c>
+      <c r="W152" s="72">
+        <f>W117/(Statement!W49/Statement!W75)</f>
+        <v>2.1289400567510048</v>
+      </c>
+      <c r="X152" s="72">
+        <f>X117/(Statement!X49/Statement!X75)</f>
+        <v>2.5271669897535309</v>
+      </c>
+      <c r="Y152" s="72">
+        <f>Y117/(Statement!Y49/Statement!Y75)</f>
+        <v>4.408950787334625</v>
+      </c>
+      <c r="Z152" s="72">
+        <f>Z117/(Statement!Z49/Statement!Z75)</f>
+        <v>6.4691988572848098</v>
+      </c>
+      <c r="AA152" s="72">
+        <f>AA117/(Statement!AA49/Statement!AA75)</f>
+        <v>10.351595250387197</v>
+      </c>
       <c r="AC152" s="72">
         <f ca="1">AC117/(Statement!AC49/Statement!AC75)</f>
-        <v>9.5157514594336998</v>
+        <v>9.2252181208053692</v>
       </c>
     </row>
     <row r="153" spans="2:29" x14ac:dyDescent="0.2">
@@ -34005,17 +34069,41 @@
         <f>Statement!Q117*Statement!Q78</f>
         <v>137982</v>
       </c>
-      <c r="T153" s="49"/>
-      <c r="U153" s="49"/>
-      <c r="V153" s="49"/>
-      <c r="W153" s="49"/>
-      <c r="X153" s="49"/>
-      <c r="Y153" s="49"/>
-      <c r="Z153" s="49"/>
-      <c r="AA153" s="49"/>
+      <c r="T153" s="147">
+        <f>Statement!T117*Statement!T78</f>
+        <v>107229.54</v>
+      </c>
+      <c r="U153" s="147">
+        <f>Statement!U117*Statement!U78</f>
+        <v>109912.5</v>
+      </c>
+      <c r="V153" s="147">
+        <f>Statement!V117*Statement!V78</f>
+        <v>103389.31999999999</v>
+      </c>
+      <c r="W153" s="147">
+        <f>Statement!W117*Statement!W78</f>
+        <v>108715.3</v>
+      </c>
+      <c r="X153" s="147">
+        <f>Statement!X117*Statement!X78</f>
+        <v>137982</v>
+      </c>
+      <c r="Y153" s="147">
+        <f>Statement!Y117*Statement!Y78</f>
+        <v>262266.14</v>
+      </c>
+      <c r="Z153" s="147">
+        <f>Statement!Z117*Statement!Z78</f>
+        <v>475400.64</v>
+      </c>
+      <c r="AA153" s="147">
+        <f>Statement!AA117*Statement!AA78</f>
+        <v>1058353.92</v>
+      </c>
       <c r="AC153" s="147">
         <f ca="1">Statement!AC117*Statement!AC78</f>
-        <v>972896.70000000007</v>
+        <v>943192.38</v>
       </c>
     </row>
     <row r="154" spans="2:29" x14ac:dyDescent="0.2">
@@ -34042,17 +34130,41 @@
         <f>Q153+Q108-Q107+Q48+Q45</f>
         <v>140623</v>
       </c>
-      <c r="T154" s="49"/>
-      <c r="U154" s="49"/>
-      <c r="V154" s="49"/>
-      <c r="W154" s="49"/>
-      <c r="X154" s="49"/>
-      <c r="Y154" s="49"/>
-      <c r="Z154" s="49"/>
-      <c r="AA154" s="49"/>
+      <c r="T154" s="147">
+        <f t="shared" ref="T154:AA154" si="99">T153+T108-T107+T48+T45</f>
+        <v>111474.54</v>
+      </c>
+      <c r="U154" s="147">
+        <f t="shared" si="99"/>
+        <v>114953.5</v>
+      </c>
+      <c r="V154" s="147">
+        <f t="shared" si="99"/>
+        <v>108154.31999999999</v>
+      </c>
+      <c r="W154" s="147">
+        <f t="shared" si="99"/>
+        <v>112043.3</v>
+      </c>
+      <c r="X154" s="147">
+        <f t="shared" si="99"/>
+        <v>140623</v>
+      </c>
+      <c r="Y154" s="147">
+        <f t="shared" si="99"/>
+        <v>262007.14</v>
+      </c>
+      <c r="Z154" s="147">
+        <f t="shared" si="99"/>
+        <v>468915.64</v>
+      </c>
+      <c r="AA154" s="147">
+        <f t="shared" si="99"/>
+        <v>1033947.9199999999</v>
+      </c>
       <c r="AC154" s="147">
         <f ca="1">AC153+AC108-AC107+AC48+AC45</f>
-        <v>948490.70000000007</v>
+        <v>918786.38</v>
       </c>
     </row>
     <row r="155" spans="2:29" x14ac:dyDescent="0.2">
@@ -34089,7 +34201,7 @@
       <c r="AA155" s="49"/>
       <c r="AC155" s="187">
         <f ca="1">AC154/AC5</f>
-        <v>10.506798192170503</v>
+        <v>10.177751955158739</v>
       </c>
     </row>
     <row r="156" spans="2:29" x14ac:dyDescent="0.2">
@@ -34126,7 +34238,7 @@
       <c r="AA156" s="49"/>
       <c r="AC156" s="187">
         <f ca="1">AC154/AC12</f>
-        <v>16.010173353813954</v>
+        <v>15.508775382745641</v>
       </c>
     </row>
     <row r="157" spans="2:29" x14ac:dyDescent="0.2">
@@ -34154,35 +34266,35 @@
         <v>696</v>
       </c>
       <c r="T157" s="64">
-        <f t="shared" ref="T157:AA157" si="98">T59-T54+T110+T65</f>
+        <f t="shared" ref="T157:AA157" si="100">T59-T54+T110+T65</f>
         <v>0</v>
       </c>
       <c r="U157" s="64">
-        <f t="shared" si="98"/>
+        <f t="shared" si="100"/>
         <v>-182</v>
       </c>
       <c r="V157" s="64">
-        <f t="shared" si="98"/>
+        <f t="shared" si="100"/>
         <v>-362</v>
       </c>
       <c r="W157" s="64">
-        <f t="shared" si="98"/>
+        <f t="shared" si="100"/>
         <v>1418</v>
       </c>
       <c r="X157" s="64">
-        <f t="shared" si="98"/>
+        <f t="shared" si="100"/>
         <v>-178</v>
       </c>
       <c r="Y157" s="64">
-        <f t="shared" si="98"/>
+        <f t="shared" si="100"/>
         <v>2732</v>
       </c>
       <c r="Z157" s="64">
-        <f t="shared" si="98"/>
+        <f t="shared" si="100"/>
         <v>5207</v>
       </c>
       <c r="AA157" s="64">
-        <f t="shared" si="98"/>
+        <f t="shared" si="100"/>
         <v>17207</v>
       </c>
       <c r="AC157" s="64">
@@ -34236,19 +34348,19 @@
         <v>46.109126213592226</v>
       </c>
       <c r="N159" s="72">
-        <f t="shared" ref="N159:Q159" si="99">N153/N157</f>
+        <f t="shared" ref="N159:Q159" si="101">N153/N157</f>
         <v>24.180411538461538</v>
       </c>
       <c r="O159" s="72">
-        <f t="shared" si="99"/>
+        <f t="shared" si="101"/>
         <v>-11.137020706092658</v>
       </c>
       <c r="P159" s="72">
-        <f t="shared" si="99"/>
+        <f t="shared" si="101"/>
         <v>-150.60328651685393</v>
       </c>
       <c r="Q159" s="72">
-        <f t="shared" si="99"/>
+        <f t="shared" si="101"/>
         <v>198.25</v>
       </c>
       <c r="T159" s="49"/>
@@ -34260,8 +34372,8 @@
       <c r="Z159" s="49"/>
       <c r="AA159" s="49"/>
       <c r="AC159" s="72">
-        <f t="shared" ref="AC159:AC160" ca="1" si="100">AC153/AC157</f>
-        <v>38.965744152515221</v>
+        <f t="shared" ref="AC159:AC160" ca="1" si="102">AC153/AC157</f>
+        <v>37.776048542133928</v>
       </c>
     </row>
     <row r="160" spans="2:29" x14ac:dyDescent="0.2">
@@ -34273,19 +34385,19 @@
         <v>53.778212366868843</v>
       </c>
       <c r="N160" s="72">
-        <f t="shared" ref="N160:Q160" si="101">N154/N158</f>
+        <f t="shared" ref="N160:Q160" si="103">N154/N158</f>
         <v>22.563526344447098</v>
       </c>
       <c r="O160" s="72">
-        <f t="shared" si="101"/>
+        <f t="shared" si="103"/>
         <v>-9.0750052588524017</v>
       </c>
       <c r="P160" s="72">
-        <f t="shared" si="101"/>
+        <f t="shared" si="103"/>
         <v>-168.8298535317509</v>
       </c>
       <c r="Q160" s="72">
-        <f t="shared" si="101"/>
+        <f t="shared" si="103"/>
         <v>178.11781476710598</v>
       </c>
       <c r="T160" s="49"/>
@@ -34297,8 +34409,8 @@
       <c r="Z160" s="49"/>
       <c r="AA160" s="49"/>
       <c r="AC160" s="72">
-        <f t="shared" ca="1" si="100"/>
-        <v>38.357082656680674</v>
+        <f t="shared" ca="1" si="102"/>
+        <v>37.155836236973563</v>
       </c>
     </row>
     <row r="161" spans="2:29" x14ac:dyDescent="0.2">
@@ -34310,19 +34422,19 @@
         <v>2.1687680555204626E-2</v>
       </c>
       <c r="N161" s="74">
-        <f t="shared" ref="N161:Q161" si="102">N157/N153</f>
+        <f t="shared" ref="N161:Q161" si="104">N157/N153</f>
         <v>4.1355789102654132E-2</v>
       </c>
       <c r="O161" s="74">
-        <f t="shared" si="102"/>
+        <f t="shared" si="104"/>
         <v>-8.9790620525014964E-2</v>
       </c>
       <c r="P161" s="74">
-        <f t="shared" si="102"/>
+        <f t="shared" si="104"/>
         <v>-6.6399613390116198E-3</v>
       </c>
       <c r="Q161" s="74">
-        <f t="shared" si="102"/>
+        <f t="shared" si="104"/>
         <v>5.0441361916771753E-3</v>
       </c>
       <c r="T161" s="49"/>
@@ -34334,8 +34446,8 @@
       <c r="Z161" s="49"/>
       <c r="AA161" s="49"/>
       <c r="AC161" s="74">
-        <f t="shared" ref="AC161" ca="1" si="103">AC157/AC153</f>
-        <v>2.5663567365373938E-2</v>
+        <f t="shared" ref="AC161" ca="1" si="105">AC157/AC153</f>
+        <v>2.6471799952412677E-2</v>
       </c>
     </row>
     <row r="162" spans="2:29" x14ac:dyDescent="0.2">
@@ -34372,7 +34484,7 @@
       <c r="AA162" s="49"/>
       <c r="AC162" s="74">
         <f ca="1">AC26/AC117</f>
-        <v>5.2028976971553093E-2</v>
+        <v>5.3667545532969638E-2</v>
       </c>
     </row>
     <row r="163" spans="2:29" x14ac:dyDescent="0.2">
@@ -34409,7 +34521,7 @@
       <c r="AA163" s="49"/>
       <c r="AC163" s="158">
         <f ca="1">AC82/AC117</f>
-        <v>6.2430060663172158E-4</v>
+        <v>6.4396194549408892E-4</v>
       </c>
     </row>
     <row r="164" spans="2:29" x14ac:dyDescent="0.2">
@@ -34446,7 +34558,7 @@
       <c r="AA164" s="49"/>
       <c r="AC164" s="158">
         <f ca="1">-AC63/AC153</f>
-        <v>1.1532570724106679E-3</v>
+        <v>1.1895770404760904E-3</v>
       </c>
     </row>
     <row r="165" spans="2:29" x14ac:dyDescent="0.2">
@@ -34483,7 +34595,7 @@
       <c r="AA165" s="49"/>
       <c r="AC165" s="158">
         <f ca="1">-(AC63+AC64)/AC153</f>
-        <v>1.7360527587358451E-3</v>
+        <v>1.790726935262136E-3</v>
       </c>
     </row>
     <row r="166" spans="2:29" x14ac:dyDescent="0.2">
@@ -34733,35 +34845,35 @@
         <v>10.638146167557933</v>
       </c>
       <c r="T172" s="72">
-        <f t="shared" ref="T172:AA172" si="104">T107/T75</f>
+        <f t="shared" ref="T172:AA172" si="106">T107/T75</f>
         <v>8.252479711451759</v>
       </c>
       <c r="U172" s="72">
-        <f t="shared" si="104"/>
+        <f t="shared" si="106"/>
         <v>7.8491921005386001</v>
       </c>
       <c r="V172" s="72">
-        <f t="shared" si="104"/>
+        <f t="shared" si="106"/>
         <v>8.5778175313059037</v>
       </c>
       <c r="W172" s="72">
-        <f t="shared" si="104"/>
+        <f t="shared" si="106"/>
         <v>10.914209115281501</v>
       </c>
       <c r="X172" s="72">
-        <f t="shared" si="104"/>
+        <f t="shared" si="106"/>
         <v>10.638146167557933</v>
       </c>
       <c r="Y172" s="72">
-        <f t="shared" si="104"/>
+        <f t="shared" si="106"/>
         <v>10.670515097690942</v>
       </c>
       <c r="Z172" s="72">
-        <f t="shared" si="104"/>
+        <f t="shared" si="106"/>
         <v>14.740248226950355</v>
       </c>
       <c r="AA172" s="72">
-        <f t="shared" si="104"/>
+        <f t="shared" si="106"/>
         <v>26.685562444641274</v>
       </c>
       <c r="AC172" s="72">
@@ -34794,35 +34906,35 @@
         <v>5.5463623395149785E-2</v>
       </c>
       <c r="T173" s="158" t="e">
-        <f t="shared" ref="T173:AA173" si="105">T54/T59</f>
+        <f t="shared" ref="T173:AA173" si="107">T54/T59</f>
         <v>#DIV/0!</v>
       </c>
       <c r="U173" s="158">
-        <f t="shared" si="105"/>
+        <f t="shared" si="107"/>
         <v>6.7817509247842175E-2</v>
       </c>
       <c r="V173" s="158">
-        <f t="shared" si="105"/>
+        <f t="shared" si="107"/>
         <v>6.3165905631659053E-2</v>
       </c>
       <c r="W173" s="158">
-        <f t="shared" si="105"/>
+        <f t="shared" si="107"/>
         <v>5.4892601431980909E-2</v>
       </c>
       <c r="X173" s="158">
-        <f t="shared" si="105"/>
+        <f t="shared" si="107"/>
         <v>4.3630017452006981E-2</v>
       </c>
       <c r="Y173" s="158">
-        <f t="shared" si="105"/>
+        <f t="shared" si="107"/>
         <v>3.4478658899060752E-2</v>
       </c>
       <c r="Z173" s="158">
-        <f t="shared" si="105"/>
+        <f t="shared" si="107"/>
         <v>2.5959842056624379E-2</v>
       </c>
       <c r="AA173" s="158">
-        <f t="shared" si="105"/>
+        <f t="shared" si="107"/>
         <v>1.3982984086970221E-2</v>
       </c>
       <c r="AC173" s="158">
@@ -34855,35 +34967,35 @@
         <v>2.600460163732677E-2</v>
       </c>
       <c r="T174" s="158">
-        <f t="shared" ref="T174:AA174" si="106">T54/T5</f>
+        <f t="shared" ref="T174:AA174" si="108">T54/T5</f>
         <v>0</v>
       </c>
       <c r="U174" s="158">
-        <f t="shared" si="106"/>
+        <f t="shared" si="108"/>
         <v>2.5261224021127571E-2</v>
       </c>
       <c r="V174" s="158">
-        <f t="shared" si="106"/>
+        <f t="shared" si="108"/>
         <v>3.0920153979883274E-2</v>
       </c>
       <c r="W174" s="158">
-        <f t="shared" si="106"/>
+        <f t="shared" si="108"/>
         <v>2.7201376196107945E-2</v>
       </c>
       <c r="X174" s="158">
-        <f t="shared" si="106"/>
+        <f t="shared" si="108"/>
         <v>2.209456473707468E-2</v>
       </c>
       <c r="Y174" s="158">
-        <f t="shared" si="106"/>
+        <f t="shared" si="108"/>
         <v>2.1256321923330646E-2</v>
       </c>
       <c r="Z174" s="158">
-        <f t="shared" si="106"/>
+        <f t="shared" si="108"/>
         <v>1.2950544844928752E-2</v>
       </c>
       <c r="AA174" s="158">
-        <f t="shared" si="106"/>
+        <f t="shared" si="108"/>
         <v>8.5632960247008869E-3</v>
       </c>
       <c r="AC174" s="158">
@@ -34916,35 +35028,35 @@
         <v>-2.3538324420677363</v>
       </c>
       <c r="T175" s="72">
-        <f t="shared" ref="T175:AA175" si="107">(T107-T108)/T75</f>
+        <f t="shared" ref="T175:AA175" si="109">(T107-T108)/T75</f>
         <v>-3.8277727682596936</v>
       </c>
       <c r="U175" s="72">
-        <f t="shared" si="107"/>
+        <f t="shared" si="109"/>
         <v>-4.5251346499102336</v>
       </c>
       <c r="V175" s="72">
-        <f t="shared" si="107"/>
+        <f t="shared" si="109"/>
         <v>-4.2620751341681578</v>
       </c>
       <c r="W175" s="72">
-        <f t="shared" si="107"/>
+        <f t="shared" si="109"/>
         <v>-2.9740840035746201</v>
       </c>
       <c r="X175" s="72">
-        <f t="shared" si="107"/>
+        <f t="shared" si="109"/>
         <v>-2.3538324420677363</v>
       </c>
       <c r="Y175" s="72">
-        <f t="shared" si="107"/>
+        <f t="shared" si="109"/>
         <v>0.23001776198934282</v>
       </c>
       <c r="Z175" s="72">
-        <f t="shared" si="107"/>
+        <f t="shared" si="109"/>
         <v>5.749113475177305</v>
       </c>
       <c r="AA175" s="72">
-        <f t="shared" si="107"/>
+        <f t="shared" si="109"/>
         <v>21.617360496014172</v>
       </c>
       <c r="AC175" s="72">
@@ -34986,7 +35098,7 @@
       <c r="AA176" s="49"/>
       <c r="AC176" s="158">
         <f ca="1">(AC107-AC108)/AC153</f>
-        <v>2.5085910970815296E-2</v>
+        <v>2.5875951203083298E-2</v>
       </c>
     </row>
     <row r="177" spans="1:31" x14ac:dyDescent="0.2">
@@ -35014,35 +35126,35 @@
         <v>0.42423350634062817</v>
       </c>
       <c r="T177" s="158">
-        <f t="shared" ref="T177:AA177" si="108">-T110/T5</f>
+        <f t="shared" ref="T177:AA177" si="110">-T110/T5</f>
         <v>0</v>
       </c>
       <c r="U177" s="158">
-        <f t="shared" si="108"/>
+        <f t="shared" si="110"/>
         <v>0.36812492823515902</v>
       </c>
       <c r="V177" s="158">
-        <f t="shared" si="108"/>
+        <f t="shared" si="110"/>
         <v>0.50353905376878183</v>
       </c>
       <c r="W177" s="158">
-        <f t="shared" si="108"/>
+        <f t="shared" si="110"/>
         <v>0.31588001290183854</v>
       </c>
       <c r="X177" s="158">
-        <f t="shared" si="108"/>
+        <f t="shared" si="110"/>
         <v>0.50004418912947413</v>
       </c>
       <c r="Y177" s="158">
-        <f t="shared" si="108"/>
+        <f t="shared" si="110"/>
         <v>0.39500109946492706</v>
       </c>
       <c r="Z177" s="158">
-        <f t="shared" si="108"/>
+        <f t="shared" si="110"/>
         <v>0.26768650461022631</v>
       </c>
       <c r="AA177" s="158">
-        <f t="shared" si="108"/>
+        <f t="shared" si="110"/>
         <v>0.18877846391354688</v>
       </c>
       <c r="AC177" s="158">
@@ -35075,35 +35187,35 @@
         <v>0.90482168330955781</v>
       </c>
       <c r="T178" s="158" t="e">
-        <f t="shared" ref="T178:AA178" si="109">-(T110/T59)</f>
+        <f t="shared" ref="T178:AA178" si="111">-(T110/T59)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="U178" s="158">
-        <f t="shared" si="109"/>
+        <f t="shared" si="111"/>
         <v>0.98828606658446361</v>
       </c>
       <c r="V178" s="158">
-        <f t="shared" si="109"/>
+        <f t="shared" si="111"/>
         <v>1.0286656519533233</v>
       </c>
       <c r="W178" s="158">
-        <f t="shared" si="109"/>
+        <f t="shared" si="111"/>
         <v>0.6374484703840313</v>
       </c>
       <c r="X178" s="158">
-        <f t="shared" si="109"/>
+        <f t="shared" si="111"/>
         <v>0.98743455497382204</v>
       </c>
       <c r="Y178" s="158">
-        <f t="shared" si="109"/>
+        <f t="shared" si="111"/>
         <v>0.64070859588633933</v>
       </c>
       <c r="Z178" s="158">
-        <f t="shared" si="109"/>
+        <f t="shared" si="111"/>
         <v>0.53658741493741069</v>
       </c>
       <c r="AA178" s="158">
-        <f t="shared" si="109"/>
+        <f t="shared" si="111"/>
         <v>0.30825586891444778</v>
       </c>
       <c r="AC178" s="158">
@@ -35136,35 +35248,35 @@
         <v>1.8985871647509578</v>
       </c>
       <c r="T179" s="158" t="e">
-        <f t="shared" ref="T179:AA179" si="110">-T110/T53</f>
+        <f t="shared" ref="T179:AA179" si="112">-T110/T53</f>
         <v>#DIV/0!</v>
       </c>
       <c r="U179" s="158">
-        <f t="shared" si="110"/>
+        <f t="shared" si="112"/>
         <v>1.5793103448275863</v>
       </c>
       <c r="V179" s="158">
-        <f t="shared" si="110"/>
+        <f t="shared" si="112"/>
         <v>1.9504569504569504</v>
       </c>
       <c r="W179" s="158">
-        <f t="shared" si="110"/>
+        <f t="shared" si="112"/>
         <v>1.4030563514804202</v>
       </c>
       <c r="X179" s="158">
-        <f t="shared" si="110"/>
+        <f t="shared" si="112"/>
         <v>2.6328524895300141</v>
       </c>
       <c r="Y179" s="158">
-        <f t="shared" si="110"/>
+        <f t="shared" si="112"/>
         <v>2.4362567811934901</v>
       </c>
       <c r="Z179" s="158">
-        <f t="shared" si="110"/>
+        <f t="shared" si="112"/>
         <v>2.7939632545931761</v>
       </c>
       <c r="AA179" s="158">
-        <f t="shared" si="110"/>
+        <f t="shared" si="112"/>
         <v>3.3104906937394247</v>
       </c>
       <c r="AC179" s="158">
@@ -35181,19 +35293,19 @@
         <v>0.47078115176128738</v>
       </c>
       <c r="N180" s="228">
-        <f t="shared" ref="N180:Q180" si="111">N5/N37</f>
+        <f t="shared" ref="N180:Q180" si="113">N5/N37</f>
         <v>0.4640405533847291</v>
       </c>
       <c r="O180" s="228">
-        <f t="shared" si="111"/>
+        <f t="shared" si="113"/>
         <v>0.24185264730600431</v>
       </c>
       <c r="P180" s="228">
-        <f t="shared" si="111"/>
+        <f t="shared" si="113"/>
         <v>0.36174657139564365</v>
       </c>
       <c r="Q180" s="228">
-        <f t="shared" si="111"/>
+        <f t="shared" si="113"/>
         <v>0.45143602502475905</v>
       </c>
       <c r="T180" s="49"/>
@@ -35205,7 +35317,7 @@
       <c r="Z180" s="49"/>
       <c r="AA180" s="49"/>
       <c r="AC180" s="228">
-        <f t="shared" ref="AC180" si="112">AC5/AC37</f>
+        <f t="shared" ref="AC180" si="114">AC5/AC37</f>
         <v>0.67312395609639708</v>
       </c>
     </row>
@@ -35218,19 +35330,19 @@
         <v>1.0784657010982015</v>
       </c>
       <c r="N181" s="230">
-        <f t="shared" ref="N181:Q181" si="113">IF(AND(N12&gt;0,N108&gt;0),N108/N12,"N/A")</f>
+        <f t="shared" ref="N181:Q181" si="115">IF(AND(N12&gt;0,N108&gt;0),N108/N12,"N/A")</f>
         <v>0.71181199752628321</v>
       </c>
       <c r="O181" s="230" t="str">
-        <f t="shared" si="113"/>
+        <f t="shared" si="115"/>
         <v>N/A</v>
       </c>
       <c r="P181" s="230">
-        <f t="shared" si="113"/>
+        <f t="shared" si="115"/>
         <v>10.27377300613497</v>
       </c>
       <c r="Q181" s="230">
-        <f t="shared" si="113"/>
+        <f t="shared" si="115"/>
         <v>1.4920163766632548</v>
       </c>
       <c r="T181" s="49"/>
@@ -35242,7 +35354,7 @@
       <c r="Z181" s="49"/>
       <c r="AA181" s="49"/>
       <c r="AC181" s="230">
-        <f t="shared" ref="AC181" si="114">IF(AND(AC12&gt;0,AC108&gt;0),AC108/AC12,"N/A")</f>
+        <f t="shared" ref="AC181" si="116">IF(AND(AC12&gt;0,AC108&gt;0),AC108/AC12,"N/A")</f>
         <v>9.6585250578127377E-2</v>
       </c>
     </row>
@@ -35255,19 +35367,19 @@
         <v>-0.57647620563425117</v>
       </c>
       <c r="N182" s="230">
-        <f t="shared" ref="N182:Q182" si="115">IF(AND(N12&gt;0,N108&gt;0),(N108-N107)/N12,"N/A")</f>
+        <f t="shared" ref="N182:Q182" si="117">IF(AND(N12&gt;0,N108&gt;0),(N108-N107)/N12,"N/A")</f>
         <v>-0.41970727685013398</v>
       </c>
       <c r="O182" s="230" t="str">
-        <f t="shared" si="115"/>
+        <f t="shared" si="117"/>
         <v>N/A</v>
       </c>
       <c r="P182" s="230">
-        <f t="shared" si="115"/>
+        <f t="shared" si="117"/>
         <v>3.2553680981595092</v>
       </c>
       <c r="Q182" s="230">
-        <f t="shared" si="115"/>
+        <f t="shared" si="117"/>
         <v>0.27031729785056297</v>
       </c>
       <c r="T182" s="49"/>
@@ -35279,7 +35391,7 @@
       <c r="Z182" s="49"/>
       <c r="AA182" s="49"/>
       <c r="AC182" s="230">
-        <f t="shared" ref="AC182" si="116">IF(AND(AC12&gt;0,AC108&gt;0),(AC108-AC107)/AC12,"N/A")</f>
+        <f t="shared" ref="AC182" si="118">IF(AND(AC12&gt;0,AC108&gt;0),(AC108-AC107)/AC12,"N/A")</f>
         <v>-0.41196428270006585</v>
       </c>
     </row>
@@ -35292,19 +35404,19 @@
         <v>0.68728138721440801</v>
       </c>
       <c r="N183" s="230">
-        <f t="shared" ref="N183:Q183" si="117">N5/(N108+N112-N107)</f>
+        <f t="shared" ref="N183:Q183" si="119">N5/(N108+N112-N107)</f>
         <v>0.67105923420966507</v>
       </c>
       <c r="O183" s="230">
-        <f t="shared" si="117"/>
+        <f t="shared" si="119"/>
         <v>0.33055390113162597</v>
       </c>
       <c r="P183" s="230">
-        <f t="shared" si="117"/>
+        <f t="shared" si="119"/>
         <v>0.50856691510045371</v>
       </c>
       <c r="Q183" s="230">
-        <f t="shared" si="117"/>
+        <f t="shared" si="119"/>
         <v>0.65799387388656128</v>
       </c>
       <c r="T183" s="49"/>
@@ -35316,7 +35428,7 @@
       <c r="Z183" s="49"/>
       <c r="AA183" s="49"/>
       <c r="AC183" s="230">
-        <f t="shared" ref="AC183" si="118">AC5/(AC108+AC112-AC107)</f>
+        <f t="shared" ref="AC183" si="120">AC5/(AC108+AC112-AC107)</f>
         <v>1.1828664273172778</v>
       </c>
     </row>
@@ -35450,7 +35562,7 @@
         <v>9943</v>
       </c>
       <c r="AC188" s="62">
-        <f t="shared" ref="AC188:AC199" si="119">SUM(X188:AA188)</f>
+        <f t="shared" ref="AC188:AC199" si="121">SUM(X188:AA188)</f>
         <v>23945</v>
       </c>
     </row>
@@ -35510,7 +35622,7 @@
         <v>185</v>
       </c>
       <c r="AC189" s="62">
-        <f t="shared" si="119"/>
+        <f t="shared" si="121"/>
         <v>597</v>
       </c>
     </row>
@@ -35583,7 +35695,7 @@
         <v>13769</v>
       </c>
       <c r="AC191" s="62">
-        <f t="shared" si="119"/>
+        <f t="shared" si="121"/>
         <v>31345</v>
       </c>
     </row>
@@ -35641,7 +35753,7 @@
         <v>11524</v>
       </c>
       <c r="AC192" s="62">
-        <f t="shared" si="119"/>
+        <f t="shared" si="121"/>
         <v>21167</v>
       </c>
     </row>
@@ -35699,7 +35811,7 @@
         <v>11521</v>
       </c>
       <c r="AC193" s="62">
-        <f t="shared" si="119"/>
+        <f t="shared" si="121"/>
         <v>27247</v>
       </c>
     </row>
@@ -35757,7 +35869,7 @@
         <v>4634</v>
       </c>
       <c r="AC194" s="62">
-        <f t="shared" si="119"/>
+        <f t="shared" si="121"/>
         <v>10496</v>
       </c>
     </row>
@@ -35841,7 +35953,7 @@
         <v>2278</v>
       </c>
       <c r="AC196" s="62">
-        <f t="shared" si="119"/>
+        <f t="shared" si="121"/>
         <v>7939</v>
       </c>
     </row>
@@ -35899,7 +36011,7 @@
         <v>1537</v>
       </c>
       <c r="AC197" s="62">
-        <f t="shared" si="119"/>
+        <f t="shared" si="121"/>
         <v>5078</v>
       </c>
     </row>
@@ -35957,7 +36069,7 @@
         <v>1463</v>
       </c>
       <c r="AC198" s="62">
-        <f t="shared" si="119"/>
+        <f t="shared" si="121"/>
         <v>7480</v>
       </c>
     </row>
@@ -36015,7 +36127,7 @@
         <v>975</v>
       </c>
       <c r="AC199" s="62">
-        <f t="shared" si="119"/>
+        <f t="shared" si="121"/>
         <v>3763</v>
       </c>
     </row>
@@ -36080,179 +36192,179 @@
       <c r="K203" s="81"/>
       <c r="L203" s="81"/>
       <c r="M203" s="81">
-        <f t="shared" ref="M203:Q210" si="120">IF(L187=0,
+        <f t="shared" ref="M203:Q210" si="122">IF(L187=0,
 IF(M187=0,0,IF(M187&gt;0,1,-1)),
 (M187-L187)/ABS(L187)
 )</f>
         <v>1</v>
       </c>
       <c r="N203" s="81">
-        <f t="shared" si="120"/>
+        <f t="shared" si="122"/>
         <v>0.11712161285493287</v>
       </c>
       <c r="O203" s="81">
-        <f t="shared" si="120"/>
+        <f t="shared" si="122"/>
         <v>-0.5096042169212901</v>
       </c>
       <c r="P203" s="81">
-        <f t="shared" si="120"/>
+        <f t="shared" si="122"/>
         <v>0.60347968664601936</v>
       </c>
       <c r="Q203" s="81">
-        <f t="shared" si="120"/>
+        <f t="shared" si="122"/>
         <v>0.62347327160143162</v>
       </c>
       <c r="T203" s="81">
-        <f t="shared" ref="T203:AA205" si="121">IF(S187=0,
+        <f t="shared" ref="T203:AA205" si="123">IF(S187=0,
 IF(T187=0,0,IF(T187&gt;0,1,-1)),
 (T187-S187)/ABS(S187)
 )</f>
         <v>1</v>
       </c>
       <c r="U203" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>-0.54853273137697522</v>
       </c>
       <c r="V203" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>-4.328125E-2</v>
       </c>
       <c r="W203" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>0.15482606565409113</v>
       </c>
       <c r="X203" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>2.1364729175505586</v>
       </c>
       <c r="Y203" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>-0.51248985481107401</v>
       </c>
       <c r="Z203" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>0.73584905660377353</v>
       </c>
       <c r="AA203" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>0.66922421142369992</v>
       </c>
       <c r="AC203" s="49"/>
     </row>
     <row r="204" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B204" s="20" t="str">
-        <f t="shared" ref="B204:B210" si="122">B188</f>
+        <f t="shared" ref="B204:B210" si="124">B188</f>
         <v>NAND</v>
       </c>
       <c r="M204" s="81">
-        <f t="shared" si="120"/>
+        <f t="shared" si="122"/>
         <v>1</v>
       </c>
       <c r="N204" s="81">
-        <f t="shared" si="120"/>
+        <f t="shared" si="122"/>
         <v>0.11474240045668617</v>
       </c>
       <c r="O204" s="81">
-        <f t="shared" si="120"/>
+        <f t="shared" si="122"/>
         <v>-0.46152861349379082</v>
       </c>
       <c r="P204" s="81">
-        <f t="shared" si="120"/>
+        <f t="shared" si="122"/>
         <v>0.71825962910128383</v>
       </c>
       <c r="Q204" s="81">
-        <f t="shared" si="120"/>
+        <f t="shared" si="122"/>
         <v>0.17656012176560121</v>
       </c>
       <c r="T204" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>1</v>
       </c>
       <c r="U204" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>-0.62631315657828912</v>
       </c>
       <c r="V204" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>-0.17224453369031684</v>
       </c>
       <c r="W204" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>0.16172506738544473</v>
       </c>
       <c r="X204" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>1.9058004640371229</v>
       </c>
       <c r="Y204" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>-0.56196103481315873</v>
       </c>
       <c r="Z204" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>0.82172803499817715</v>
       </c>
       <c r="AA204" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>0.98979387632579552</v>
       </c>
       <c r="AC204" s="49"/>
     </row>
     <row r="205" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B205" s="20" t="str">
+        <f t="shared" si="124"/>
+        <v>Other</v>
+      </c>
+      <c r="M205" s="81">
         <f t="shared" si="122"/>
-        <v>Other</v>
-      </c>
-      <c r="M205" s="81">
-        <f t="shared" si="120"/>
         <v>1</v>
       </c>
       <c r="N205" s="81">
-        <f t="shared" si="120"/>
+        <f t="shared" si="122"/>
         <v>-0.14871016691957512</v>
       </c>
       <c r="O205" s="81">
-        <f t="shared" si="120"/>
+        <f t="shared" si="122"/>
         <v>-0.36541889483065954</v>
       </c>
       <c r="P205" s="81">
-        <f t="shared" si="120"/>
+        <f t="shared" si="122"/>
         <v>-0.21067415730337077</v>
       </c>
       <c r="Q205" s="81">
-        <f t="shared" si="120"/>
+        <f t="shared" si="122"/>
         <v>5.6939501779359428E-2</v>
       </c>
       <c r="T205" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>1</v>
       </c>
       <c r="U205" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>-0.67924528301886788</v>
       </c>
       <c r="V205" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>0.10294117647058823</v>
       </c>
       <c r="W205" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>0</v>
       </c>
       <c r="X205" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>2.0533333333333332</v>
       </c>
       <c r="Y205" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>-0.61572052401746724</v>
       </c>
       <c r="Z205" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>7.9545454545454544E-2</v>
       </c>
       <c r="AA205" s="81">
-        <f t="shared" si="121"/>
+        <f t="shared" si="123"/>
         <v>0.94736842105263153</v>
       </c>
       <c r="AC205" s="49"/>
@@ -36275,92 +36387,92 @@
     </row>
     <row r="207" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B207" s="20" t="str">
+        <f t="shared" si="124"/>
+        <v>Cloud Memory</v>
+      </c>
+      <c r="M207" s="81">
         <f t="shared" si="122"/>
-        <v>Cloud Memory</v>
-      </c>
-      <c r="M207" s="81">
-        <f t="shared" si="120"/>
         <v>0</v>
       </c>
       <c r="N207" s="81">
-        <f t="shared" ref="N207:N210" si="123">IF(M191=0,
+        <f t="shared" ref="N207:N210" si="125">IF(M191=0,
 IF(N191=0,0,IF(N191&gt;0,1,-1)),
 (N191-M191)/ABS(M191)
 )</f>
         <v>0</v>
       </c>
       <c r="O207" s="81">
-        <f t="shared" ref="O207:O210" si="124">IF(N191=0,
+        <f t="shared" ref="O207:O210" si="126">IF(N191=0,
 IF(O191=0,0,IF(O191&gt;0,1,-1)),
 (O191-N191)/ABS(N191)
 )</f>
         <v>1</v>
       </c>
       <c r="P207" s="81">
-        <f t="shared" ref="P207:P210" si="125">IF(O191=0,
+        <f t="shared" ref="P207:P210" si="127">IF(O191=0,
 IF(P191=0,0,IF(P191&gt;0,1,-1)),
 (P191-O191)/ABS(O191)
 )</f>
         <v>1.0256410256410255</v>
       </c>
       <c r="Q207" s="81">
-        <f t="shared" ref="Q207:Q210" si="126">IF(P191=0,
+        <f t="shared" ref="Q207:Q210" si="128">IF(P191=0,
 IF(Q191=0,0,IF(Q191&gt;0,1,-1)),
 (Q191-P191)/ABS(P191)
 )</f>
         <v>2.5664556962025316</v>
       </c>
       <c r="T207" s="81">
-        <f t="shared" ref="T207:T210" si="127">IF(S191=0,
+        <f t="shared" ref="T207:T210" si="129">IF(S191=0,
 IF(T191=0,0,IF(T191&gt;0,1,-1)),
 (T191-S191)/ABS(S191)
 )</f>
         <v>1</v>
       </c>
       <c r="U207" s="81">
-        <f t="shared" ref="U207:U210" si="128">IF(T191=0,
+        <f t="shared" ref="U207:U210" si="130">IF(T191=0,
 IF(U191=0,0,IF(U191&gt;0,1,-1)),
 (U191-T191)/ABS(T191)
 )</f>
         <v>0.83436853002070388</v>
       </c>
       <c r="V207" s="81">
-        <f t="shared" ref="V207:V210" si="129">IF(U191=0,
+        <f t="shared" ref="V207:V210" si="131">IF(U191=0,
 IF(V191=0,0,IF(V191&gt;0,1,-1)),
 (V191-U191)/ABS(U191)
 )</f>
         <v>0.10872836719337849</v>
       </c>
       <c r="W207" s="81">
-        <f t="shared" ref="W207:W210" si="130">IF(V191=0,
+        <f t="shared" ref="W207:W210" si="132">IF(V191=0,
 IF(W191=0,0,IF(W191&gt;0,1,-1)),
 (W191-V191)/ABS(V191)
 )</f>
         <v>0.14896504920257889</v>
       </c>
       <c r="X207" s="81">
-        <f t="shared" ref="X207:X210" si="131">IF(W191=0,
+        <f t="shared" ref="X207:X210" si="133">IF(W191=0,
 IF(X191=0,0,IF(X191&gt;0,1,-1)),
 (X191-W191)/ABS(W191)
 )</f>
         <v>0.34170112226816302</v>
       </c>
       <c r="Y207" s="81">
-        <f t="shared" ref="Y207:Y210" si="132">IF(X191=0,
+        <f t="shared" ref="Y207:Y210" si="134">IF(X191=0,
 IF(Y191=0,0,IF(Y191&gt;0,1,-1)),
 (Y191-X191)/ABS(X191)
 )</f>
         <v>0.16310807836231564</v>
       </c>
       <c r="Z207" s="81">
-        <f t="shared" ref="Z207:Z210" si="133">IF(Y191=0,
+        <f t="shared" ref="Z207:Z210" si="135">IF(Y191=0,
 IF(Z191=0,0,IF(Z191&gt;0,1,-1)),
 (Z191-Y191)/ABS(Y191)
 )</f>
         <v>0.46650264950794851</v>
       </c>
       <c r="AA207" s="81">
-        <f t="shared" ref="AA207:AA210" si="134">IF(Z191=0,
+        <f t="shared" ref="AA207:AA210" si="136">IF(Z191=0,
 IF(AA191=0,0,IF(AA191&gt;0,1,-1)),
 (AA191-Z191)/ABS(Z191)
 )</f>
@@ -36370,177 +36482,177 @@
     </row>
     <row r="208" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B208" s="20" t="str">
+        <f t="shared" si="124"/>
+        <v>Core Data Center</v>
+      </c>
+      <c r="M208" s="81">
         <f t="shared" si="122"/>
-        <v>Core Data Center</v>
-      </c>
-      <c r="M208" s="81">
-        <f t="shared" si="120"/>
         <v>0</v>
       </c>
       <c r="N208" s="81">
-        <f t="shared" si="123"/>
+        <f t="shared" si="125"/>
         <v>0</v>
       </c>
       <c r="O208" s="81">
-        <f t="shared" si="124"/>
+        <f t="shared" si="126"/>
         <v>1</v>
       </c>
       <c r="P208" s="81">
-        <f t="shared" si="125"/>
+        <f t="shared" si="127"/>
         <v>1.3465160075329567</v>
       </c>
       <c r="Q208" s="81">
-        <f t="shared" si="126"/>
+        <f t="shared" si="128"/>
         <v>0.4504414125200642</v>
       </c>
       <c r="T208" s="81">
-        <f t="shared" si="127"/>
+        <f t="shared" si="129"/>
         <v>1</v>
       </c>
       <c r="U208" s="81">
-        <f t="shared" si="128"/>
+        <f t="shared" si="130"/>
         <v>0.119140625</v>
       </c>
       <c r="V208" s="81">
-        <f t="shared" si="129"/>
+        <f t="shared" si="131"/>
         <v>-0.20157068062827224</v>
       </c>
       <c r="W208" s="81">
-        <f t="shared" si="130"/>
+        <f t="shared" si="132"/>
         <v>-0.16393442622950818</v>
       </c>
       <c r="X208" s="81">
-        <f t="shared" si="131"/>
+        <f t="shared" si="133"/>
         <v>3.0718954248366011E-2</v>
       </c>
       <c r="Y208" s="81">
-        <f t="shared" si="132"/>
+        <f t="shared" si="134"/>
         <v>0.50856055802155997</v>
       </c>
       <c r="Z208" s="81">
-        <f t="shared" si="133"/>
+        <f t="shared" si="135"/>
         <v>1.3905002101723414</v>
       </c>
       <c r="AA208" s="81">
-        <f t="shared" si="134"/>
+        <f t="shared" si="136"/>
         <v>1.0263759451380341</v>
       </c>
       <c r="AC208" s="49"/>
     </row>
     <row r="209" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B209" s="20" t="str">
+        <f t="shared" si="124"/>
+        <v>Mobile and Client</v>
+      </c>
+      <c r="M209" s="81">
         <f t="shared" si="122"/>
-        <v>Mobile and Client</v>
-      </c>
-      <c r="M209" s="81">
-        <f t="shared" si="120"/>
         <v>0</v>
       </c>
       <c r="N209" s="81">
-        <f t="shared" si="123"/>
+        <f t="shared" si="125"/>
         <v>0</v>
       </c>
       <c r="O209" s="81">
-        <f t="shared" si="124"/>
+        <f t="shared" si="126"/>
         <v>1</v>
       </c>
       <c r="P209" s="81">
-        <f t="shared" si="125"/>
+        <f t="shared" si="127"/>
         <v>0.57790100081146878</v>
       </c>
       <c r="Q209" s="81">
-        <f t="shared" si="126"/>
+        <f t="shared" si="128"/>
         <v>1.6456672666495243E-2</v>
       </c>
       <c r="T209" s="81">
-        <f t="shared" si="127"/>
+        <f t="shared" si="129"/>
         <v>1</v>
       </c>
       <c r="U209" s="81">
-        <f t="shared" si="128"/>
+        <f t="shared" si="130"/>
         <v>-0.13613779397151374</v>
       </c>
       <c r="V209" s="81">
-        <f t="shared" si="129"/>
+        <f t="shared" si="131"/>
         <v>-0.14263803680981596</v>
       </c>
       <c r="W209" s="81">
-        <f t="shared" si="130"/>
+        <f t="shared" si="132"/>
         <v>0.45572450805008946</v>
       </c>
       <c r="X209" s="81">
-        <f t="shared" si="131"/>
+        <f t="shared" si="133"/>
         <v>0.15514592933947774</v>
       </c>
       <c r="Y209" s="81">
-        <f t="shared" si="132"/>
+        <f t="shared" si="134"/>
         <v>0.13164893617021275</v>
       </c>
       <c r="Z209" s="81">
-        <f t="shared" si="133"/>
+        <f t="shared" si="135"/>
         <v>0.81222091656874262</v>
       </c>
       <c r="AA209" s="81">
-        <f t="shared" si="134"/>
+        <f t="shared" si="136"/>
         <v>0.49409933860718452</v>
       </c>
       <c r="AC209" s="49"/>
     </row>
     <row r="210" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B210" s="20" t="str">
+        <f t="shared" si="124"/>
+        <v>Automotive and Embedded</v>
+      </c>
+      <c r="M210" s="81">
         <f t="shared" si="122"/>
-        <v>Automotive and Embedded</v>
-      </c>
-      <c r="M210" s="81">
-        <f t="shared" si="120"/>
         <v>0</v>
       </c>
       <c r="N210" s="81">
-        <f t="shared" si="123"/>
+        <f t="shared" si="125"/>
         <v>0</v>
       </c>
       <c r="O210" s="81">
-        <f t="shared" si="124"/>
+        <f t="shared" si="126"/>
         <v>1</v>
       </c>
       <c r="P210" s="81">
-        <f t="shared" si="125"/>
+        <f t="shared" si="127"/>
         <v>0.11886929209954095</v>
       </c>
       <c r="Q210" s="81">
-        <f t="shared" si="126"/>
+        <f t="shared" si="128"/>
         <v>2.6344202116173613E-2</v>
       </c>
       <c r="T210" s="81">
-        <f t="shared" si="127"/>
+        <f t="shared" si="129"/>
         <v>1</v>
       </c>
       <c r="U210" s="81">
-        <f t="shared" si="128"/>
+        <f t="shared" si="130"/>
         <v>-5.8536585365853662E-2</v>
       </c>
       <c r="V210" s="81">
-        <f t="shared" si="129"/>
+        <f t="shared" si="131"/>
         <v>-0.10708117443868739</v>
       </c>
       <c r="W210" s="81">
-        <f t="shared" si="130"/>
+        <f t="shared" si="132"/>
         <v>8.994197292069632E-2</v>
       </c>
       <c r="X210" s="81">
-        <f t="shared" si="131"/>
+        <f t="shared" si="133"/>
         <v>0.27240461401952087</v>
       </c>
       <c r="Y210" s="81">
-        <f t="shared" si="132"/>
+        <f t="shared" si="134"/>
         <v>0.19944211994421199</v>
       </c>
       <c r="Z210" s="81">
-        <f t="shared" si="133"/>
+        <f t="shared" si="135"/>
         <v>0.57441860465116279</v>
       </c>
       <c r="AA210" s="81">
-        <f t="shared" si="134"/>
+        <f t="shared" si="136"/>
         <v>0.71122599704579026</v>
       </c>
       <c r="AC210" s="49"/>
@@ -36680,15 +36792,15 @@
         <v>68.783005280844947</v>
       </c>
       <c r="O218" s="147">
-        <f t="shared" ref="O218:Q218" si="135">100*(1+((O117-$M117)/ABS($M117)))</f>
+        <f t="shared" ref="O218:Q218" si="137">100*(1+((O117-$M117)/ABS($M117)))</f>
         <v>81.721075372059531</v>
       </c>
       <c r="P218" s="147">
-        <f t="shared" si="135"/>
+        <f t="shared" si="137"/>
         <v>114.70235237638022</v>
       </c>
       <c r="Q218" s="147">
-        <f t="shared" si="135"/>
+        <f t="shared" si="137"/>
         <v>146.42342774843974</v>
       </c>
       <c r="T218" s="49"/>
@@ -36713,15 +36825,15 @@
         <v>111.0196715394333</v>
       </c>
       <c r="O219" s="147">
-        <f t="shared" ref="O219:Q219" si="136">100*(1+((O5-$M5)/ABS($M5)))</f>
+        <f t="shared" ref="O219:Q219" si="138">100*(1+((O5-$M5)/ABS($M5)))</f>
         <v>56.090958310774234</v>
       </c>
       <c r="P219" s="147">
-        <f t="shared" si="136"/>
+        <f t="shared" si="138"/>
         <v>90.637069121097284</v>
       </c>
       <c r="Q219" s="147">
-        <f t="shared" si="136"/>
+        <f t="shared" si="138"/>
         <v>134.91427540155206</v>
       </c>
       <c r="T219" s="49"/>
@@ -36746,15 +36858,15 @@
         <v>150.77821011673151</v>
       </c>
       <c r="O220" s="147">
-        <f t="shared" ref="O220:Q220" si="137">100*(1+((O26-$M26)/ABS($M26)))</f>
+        <f t="shared" ref="O220:Q220" si="139">100*(1+((O26-$M26)/ABS($M26)))</f>
         <v>-103.89105058365762</v>
       </c>
       <c r="P220" s="147">
-        <f t="shared" si="137"/>
+        <f t="shared" si="139"/>
         <v>13.618677042801563</v>
       </c>
       <c r="Q220" s="147">
-        <f t="shared" si="137"/>
+        <f t="shared" si="139"/>
         <v>147.66536964980546</v>
       </c>
       <c r="T220" s="49"/>
@@ -36877,7 +36989,7 @@
       </c>
       <c r="C5" s="176">
         <f ca="1">Overview!C5</f>
-        <v>848.95</v>
+        <v>823.03</v>
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="136" t="s">
@@ -36893,7 +37005,7 @@
       </c>
       <c r="C6" s="177">
         <f ca="1">Statement!AC153</f>
-        <v>972896.70000000007</v>
+        <v>943192.38</v>
       </c>
       <c r="E6" s="20" t="s">
         <v>19</v>
@@ -36913,7 +37025,7 @@
       </c>
       <c r="C7" s="177">
         <f ca="1">Statement!AC154</f>
-        <v>948490.70000000007</v>
+        <v>918786.38</v>
       </c>
       <c r="E7" s="20" t="s">
         <v>30</v>
@@ -36933,7 +37045,7 @@
       </c>
       <c r="C8" s="178">
         <f ca="1">Statement!AC150</f>
-        <v>19.220058863482002</v>
+        <v>18.633235227529998</v>
       </c>
       <c r="E8" s="20" t="s">
         <v>248</v>
@@ -36953,7 +37065,7 @@
       </c>
       <c r="C9" s="178">
         <f ca="1">Statement!AC151</f>
-        <v>10.711323858475309</v>
+        <v>10.384287502492413</v>
       </c>
       <c r="E9" s="20" t="s">
         <v>249</v>
@@ -36973,7 +37085,7 @@
       </c>
       <c r="C10" s="178">
         <f ca="1">Statement!AC152</f>
-        <v>9.5157514594336998</v>
+        <v>9.2252181208053692</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>1</v>
@@ -36993,7 +37105,7 @@
       </c>
       <c r="C11" s="178">
         <f ca="1">Statement!AC155</f>
-        <v>10.506798192170503</v>
+        <v>10.177751955158739</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
@@ -37002,7 +37114,7 @@
       </c>
       <c r="C12" s="178">
         <f ca="1">Statement!AC156</f>
-        <v>16.010173353813954</v>
+        <v>15.508775382745641</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.2">
@@ -37238,7 +37350,7 @@
       </c>
       <c r="C38" s="179">
         <f ca="1">Statement!AC162</f>
-        <v>5.2028976971553093E-2</v>
+        <v>5.3667545532969638E-2</v>
       </c>
       <c r="E38" s="20" t="s">
         <v>275</v>
@@ -37254,7 +37366,7 @@
       </c>
       <c r="C39" s="219">
         <f ca="1">Statement!AC161</f>
-        <v>2.5663567365373938E-2</v>
+        <v>2.6471799952412677E-2</v>
       </c>
       <c r="E39" s="20" t="s">
         <v>277</v>
@@ -37270,7 +37382,7 @@
       </c>
       <c r="C40" s="179">
         <f ca="1">Statement!AC163</f>
-        <v>6.2430060663172158E-4</v>
+        <v>6.4396194549408892E-4</v>
       </c>
       <c r="E40" s="20" t="s">
         <v>278</v>
@@ -37286,7 +37398,7 @@
       </c>
       <c r="C41" s="179">
         <f ca="1">Statement!AC164</f>
-        <v>1.1532570724106679E-3</v>
+        <v>1.1895770404760904E-3</v>
       </c>
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.2">
@@ -37295,7 +37407,7 @@
       </c>
       <c r="C42" s="179">
         <f ca="1">Statement!AC165</f>
-        <v>1.7360527587358451E-3</v>
+        <v>1.790726935262136E-3</v>
       </c>
     </row>
     <row r="45" spans="2:6" x14ac:dyDescent="0.2">
@@ -37339,7 +37451,7 @@
       </c>
       <c r="F48" s="179">
         <f ca="1">Statement!AC176</f>
-        <v>2.5085910970815296E-2</v>
+        <v>2.5875951203083298E-2</v>
       </c>
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.2">
@@ -37518,7 +37630,7 @@
       </c>
       <c r="I6" s="176">
         <f ca="1">Statement!AC116</f>
-        <v>848.95</v>
+        <v>823.03</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -37547,7 +37659,7 @@
       </c>
       <c r="I7" s="177">
         <f ca="1">Statement!AC153</f>
-        <v>972896.70000000007</v>
+        <v>943192.38</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
@@ -37576,7 +37688,7 @@
       </c>
       <c r="I8" s="177">
         <f ca="1">Statement!AC154</f>
-        <v>948490.70000000007</v>
+        <v>918786.38</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -37605,7 +37717,7 @@
       </c>
       <c r="I9" s="178">
         <f ca="1">Statement!AC150</f>
-        <v>19.220058863482002</v>
+        <v>18.633235227529998</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
@@ -37634,7 +37746,7 @@
       </c>
       <c r="I10" s="178">
         <f ca="1">Statement!AC151</f>
-        <v>10.711323858475309</v>
+        <v>10.384287502492413</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
@@ -37663,7 +37775,7 @@
       </c>
       <c r="I11" s="178">
         <f ca="1">Statement!AC152</f>
-        <v>9.5157514594336998</v>
+        <v>9.2252181208053692</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
@@ -37692,7 +37804,7 @@
       </c>
       <c r="I12" s="178">
         <f ca="1">Statement!AC155</f>
-        <v>10.506798192170503</v>
+        <v>10.177751955158739</v>
       </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
@@ -37721,7 +37833,7 @@
       </c>
       <c r="I13" s="178">
         <f ca="1">Statement!AC156</f>
-        <v>16.010173353813954</v>
+        <v>15.508775382745641</v>
       </c>
     </row>
     <row r="15" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -38494,7 +38606,7 @@
       </c>
       <c r="I51" s="179">
         <f ca="1">Statement!AC162</f>
-        <v>5.2028976971553093E-2</v>
+        <v>5.3667545532969638E-2</v>
       </c>
     </row>
     <row r="52" spans="2:9" x14ac:dyDescent="0.2">
@@ -38523,7 +38635,7 @@
       </c>
       <c r="I52" s="179">
         <f ca="1">Statement!AC161</f>
-        <v>2.5663567365373938E-2</v>
+        <v>2.6471799952412677E-2</v>
       </c>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.2">
@@ -38552,7 +38664,7 @@
       </c>
       <c r="I53" s="179">
         <f ca="1">Statement!AC163</f>
-        <v>6.2430060663172158E-4</v>
+        <v>6.4396194549408892E-4</v>
       </c>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.2">
@@ -38581,7 +38693,7 @@
       </c>
       <c r="I54" s="179">
         <f ca="1">Statement!AC164</f>
-        <v>1.1532570724106679E-3</v>
+        <v>1.1895770404760904E-3</v>
       </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.2">
@@ -38610,7 +38722,7 @@
       </c>
       <c r="I55" s="179">
         <f ca="1">Statement!AC165</f>
-        <v>1.7360527587358451E-3</v>
+        <v>1.790726935262136E-3</v>
       </c>
     </row>
     <row r="57" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -38846,7 +38958,7 @@
       </c>
       <c r="I68" s="200">
         <f ca="1">Statement!AC176</f>
-        <v>2.5085910970815296E-2</v>
+        <v>2.5875951203083298E-2</v>
       </c>
     </row>
     <row r="70" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">

</xml_diff>